<commit_message>
Update Evecxia IPO valuation to $180M (Axsome IPO comp)
$400M was too aggressive for a pre-Phase 2 OCD company at IPO.
$180M is anchored to Axsome at IPO ($155M, 2015) — realistic
for a CNS platform with Phase 1 complete, Phase 2 enrolling.
The sharp uptick comes from Phase 2 readout, not the IPO itself.

https://claude.ai/code/session_01F1LU9jnNeXnwBrCMYLj1kM
</commit_message>
<xml_diff>
--- a/LBRX_QSBS_Evecxia_Model.xlsx
+++ b/LBRX_QSBS_Evecxia_Model.xlsx
@@ -166,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -180,11 +180,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -465,6 +493,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1056,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1077,7 +1107,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="70" t="inlineStr">
         <is>
@@ -1160,7 +1189,6 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
@@ -1232,7 +1260,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="70" t="inlineStr">
         <is>
@@ -1287,7 +1314,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="70" t="inlineStr">
         <is>
@@ -1380,7 +1406,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="70" t="inlineStr">
         <is>
@@ -1448,7 +1473,6 @@
         <v>30000000</v>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="70" t="inlineStr">
         <is>
@@ -1486,7 +1510,6 @@
         <v>46539</v>
       </c>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
@@ -1621,7 +1644,7 @@
         </is>
       </c>
       <c r="B64" s="18" t="n">
-        <v>400000000</v>
+        <v>180000000</v>
       </c>
     </row>
     <row r="65">
@@ -2021,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2043,6 +2066,16 @@
           <t>COMP SET 1: LBRX POST-PHASE 3 POSITIVE READOUT VALUATION</t>
         </is>
       </c>
+      <c r="B1" s="108" t="n"/>
+      <c r="C1" s="108" t="n"/>
+      <c r="D1" s="108" t="n"/>
+      <c r="E1" s="108" t="n"/>
+      <c r="F1" s="108" t="n"/>
+      <c r="G1" s="108" t="n"/>
+      <c r="H1" s="108" t="n"/>
+      <c r="I1" s="108" t="n"/>
+      <c r="J1" s="108" t="n"/>
+      <c r="K1" s="109" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="85" t="inlineStr">
@@ -2360,7 +2393,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="89" t="inlineStr">
         <is>
@@ -2419,13 +2451,22 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="84" t="inlineStr">
         <is>
           <t>COMP SET 2: LBRX POST-PHASE 3 NEGATIVE READOUT / FAILURE</t>
         </is>
       </c>
+      <c r="B14" s="108" t="n"/>
+      <c r="C14" s="108" t="n"/>
+      <c r="D14" s="108" t="n"/>
+      <c r="E14" s="108" t="n"/>
+      <c r="F14" s="108" t="n"/>
+      <c r="G14" s="108" t="n"/>
+      <c r="H14" s="108" t="n"/>
+      <c r="I14" s="108" t="n"/>
+      <c r="J14" s="108" t="n"/>
+      <c r="K14" s="109" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="85" t="inlineStr">
@@ -2586,7 +2627,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="89" t="inlineStr">
         <is>
@@ -2645,13 +2685,22 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="84" t="inlineStr">
         <is>
           <t>COMP SET 3: EVECXIA PRE-PHASE 2 READOUT / IPO VALUATION</t>
         </is>
       </c>
+      <c r="B24" s="108" t="n"/>
+      <c r="C24" s="108" t="n"/>
+      <c r="D24" s="108" t="n"/>
+      <c r="E24" s="108" t="n"/>
+      <c r="F24" s="108" t="n"/>
+      <c r="G24" s="108" t="n"/>
+      <c r="H24" s="108" t="n"/>
+      <c r="I24" s="108" t="n"/>
+      <c r="J24" s="108" t="n"/>
+      <c r="K24" s="109" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="85" t="inlineStr">
@@ -2816,7 +2865,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="89" t="inlineStr">
         <is>
@@ -2875,13 +2923,22 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="84" t="inlineStr">
         <is>
           <t>COMP SET 4: EVECXIA POST-PHASE 2 POSITIVE VS NEGATIVE OUTCOMES</t>
         </is>
       </c>
+      <c r="B34" s="108" t="n"/>
+      <c r="C34" s="108" t="n"/>
+      <c r="D34" s="108" t="n"/>
+      <c r="E34" s="108" t="n"/>
+      <c r="F34" s="108" t="n"/>
+      <c r="G34" s="108" t="n"/>
+      <c r="H34" s="108" t="n"/>
+      <c r="I34" s="108" t="n"/>
+      <c r="J34" s="108" t="n"/>
+      <c r="K34" s="109" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="85" t="inlineStr">
@@ -3097,7 +3154,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="89" t="inlineStr">
         <is>
@@ -3156,7 +3212,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="89" t="inlineStr">
         <is>
@@ -3215,8 +3270,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A14:K14"/>
@@ -3234,7 +3287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3252,8 +3305,13 @@
           <t>SCENARIO ANALYSIS</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="108" t="n"/>
+      <c r="C1" s="108" t="n"/>
+      <c r="D1" s="108" t="n"/>
+      <c r="E1" s="108" t="n"/>
+      <c r="F1" s="108" t="n"/>
+      <c r="G1" s="109" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="91" t="inlineStr">
         <is>
@@ -3938,14 +3996,18 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="84" t="inlineStr">
         <is>
           <t>SCENARIO S4 DETAIL: Series B + Series C Lot-by-Lot at Lock-Up</t>
         </is>
       </c>
+      <c r="B29" s="108" t="n"/>
+      <c r="C29" s="108" t="n"/>
+      <c r="D29" s="108" t="n"/>
+      <c r="E29" s="108" t="n"/>
+      <c r="F29" s="108" t="n"/>
+      <c r="G29" s="109" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="101" t="inlineStr">
@@ -4225,14 +4287,18 @@
         <v/>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="84" t="inlineStr">
         <is>
           <t>SCENARIOS S5/S6 DETAIL: §1045 Rollover → Evecxia (Two-Leg Journey)</t>
         </is>
       </c>
+      <c r="B46" s="108" t="n"/>
+      <c r="C46" s="108" t="n"/>
+      <c r="D46" s="108" t="n"/>
+      <c r="E46" s="108" t="n"/>
+      <c r="F46" s="108" t="n"/>
+      <c r="G46" s="109" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="101" t="inlineStr">
@@ -5567,7 +5633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5586,13 +5652,14 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="84" t="inlineStr">
         <is>
           <t>KEY FLAGS</t>
         </is>
       </c>
+      <c r="B3" s="108" t="n"/>
+      <c r="C3" s="109" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="90" t="inlineStr">
@@ -5638,14 +5705,18 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="84" t="inlineStr">
         <is>
           <t>SCENARIO COMPARISON</t>
         </is>
       </c>
+      <c r="B10" s="108" t="n"/>
+      <c r="C10" s="108" t="n"/>
+      <c r="D10" s="108" t="n"/>
+      <c r="E10" s="108" t="n"/>
+      <c r="F10" s="108" t="n"/>
+      <c r="G10" s="109" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="103" t="inlineStr">
@@ -5871,14 +5942,18 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="84" t="inlineStr">
         <is>
           <t>SENSITIVITY ANALYSIS: LBRX Price vs Tax Treatment</t>
         </is>
       </c>
+      <c r="B20" s="108" t="n"/>
+      <c r="C20" s="108" t="n"/>
+      <c r="D20" s="108" t="n"/>
+      <c r="E20" s="108" t="n"/>
+      <c r="F20" s="108" t="n"/>
+      <c r="G20" s="109" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="90" t="inlineStr">
@@ -5992,33 +6067,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A20:G20"/>

</xml_diff>

<commit_message>
Add Decision Matrix, Breakeven, IRR, Dilution Waterfall + fix Scenarios formulas
Major model enhancements:
- Fix all circular references in Scenarios sheet (rows 5-23)
- Add Decision Matrix sheet: probability-weighted EV for Path 2 vs Path 3,
  head-to-head comparison, probability sensitivity table
- Add Breakeven sheet: Evecxia valuation needed to match LBRX Ph3+ base,
  capital preservation threshold, valuation-to-net sensitivity
- Add After-Tax IRR comparison across all 6 scenarios in Outputs
- Add Dilution Waterfall: ownership from Series A through Phase 2 readout
- Add 2D sensitivity matrix: P(Ph2+) x Evecxia valuation in Outputs

https://claude.ai/code/session_01F1LU9jnNeXnwBrCMYLj1kM
</commit_message>
<xml_diff>
--- a/LBRX_QSBS_Evecxia_Model.xlsx
+++ b/LBRX_QSBS_Evecxia_Model.xlsx
@@ -13,8 +13,11 @@
     <sheet name="Comps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="TaxLogic" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Outputs" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Decision Matrix" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Breakeven" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dilution" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Outputs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Sources" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="fed_ltcg_rate">Inputs!$B$5</definedName>
@@ -39,15 +42,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="$#,##0.0000"/>
     <numFmt numFmtId="169" formatCode="0.00x"/>
+    <numFmt numFmtId="170" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="171" formatCode="0.0x"/>
+    <numFmt numFmtId="172" formatCode="$#,##0,,&quot;M&quot;"/>
+    <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +129,57 @@
       <name val="Calibri"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006600"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006600"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -163,6 +220,42 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+        <bgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -212,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="170">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -495,6 +588,98 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="19" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1080,6 +1265,1277 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t>OUTPUTS DASHBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="84" t="inlineStr">
+        <is>
+          <t>KEY FLAGS</t>
+        </is>
+      </c>
+      <c r="B3" s="108" t="n"/>
+      <c r="C3" s="109" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="90" t="inlineStr">
+        <is>
+          <t>QSBS 5-year met at lock-up?</t>
+        </is>
+      </c>
+      <c r="B4" s="102">
+        <f>IF(lockup_date&gt;=qsbs_5yr_date,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="90" t="inlineStr">
+        <is>
+          <t>QSBS 5-year met at Phase 3 readout?</t>
+        </is>
+      </c>
+      <c r="B5" s="102">
+        <f>IF(ph3_date&gt;=qsbs_5yr_date,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>§1045 eligible?</t>
+        </is>
+      </c>
+      <c r="B6" s="102">
+        <f>IF(AND((lockup_date-serb_date)&gt;180,Inputs!$B$33="YES"),"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="90" t="inlineStr">
+        <is>
+          <t>§1045 → §1202 chain achievable?</t>
+        </is>
+      </c>
+      <c r="B7" s="102">
+        <f>IF(AND(B6="YES",(evecxia_ph2_date-serb_date)&gt;=1826),"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="84" t="inlineStr">
+        <is>
+          <t>SCENARIO COMPARISON</t>
+        </is>
+      </c>
+      <c r="B10" s="108" t="n"/>
+      <c r="C10" s="108" t="n"/>
+      <c r="D10" s="108" t="n"/>
+      <c r="E10" s="108" t="n"/>
+      <c r="F10" s="108" t="n"/>
+      <c r="G10" s="109" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="103" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B11" s="103" t="inlineStr">
+        <is>
+          <t>S1: Lock-Up</t>
+        </is>
+      </c>
+      <c r="C11" s="103" t="inlineStr">
+        <is>
+          <t>S2: Ph3+</t>
+        </is>
+      </c>
+      <c r="D11" s="103" t="inlineStr">
+        <is>
+          <t>S3: Ph3-</t>
+        </is>
+      </c>
+      <c r="E11" s="103" t="inlineStr">
+        <is>
+          <t>S4: Dual Lot</t>
+        </is>
+      </c>
+      <c r="F11" s="103" t="inlineStr">
+        <is>
+          <t>S5: Eve+</t>
+        </is>
+      </c>
+      <c r="G11" s="103" t="inlineStr">
+        <is>
+          <t>S6: Eve-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>Gross Proceeds</t>
+        </is>
+      </c>
+      <c r="B12" s="104">
+        <f>Scenarios!B9</f>
+        <v/>
+      </c>
+      <c r="C12" s="104">
+        <f>Scenarios!C9</f>
+        <v/>
+      </c>
+      <c r="D12" s="104">
+        <f>Scenarios!D9</f>
+        <v/>
+      </c>
+      <c r="E12" s="104">
+        <f>Scenarios!D36</f>
+        <v/>
+      </c>
+      <c r="F12" s="104">
+        <f>Scenarios!F9</f>
+        <v/>
+      </c>
+      <c r="G12" s="104">
+        <f>Scenarios!G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>Gain</t>
+        </is>
+      </c>
+      <c r="B13" s="104">
+        <f>Scenarios!B11</f>
+        <v/>
+      </c>
+      <c r="C13" s="104">
+        <f>Scenarios!C11</f>
+        <v/>
+      </c>
+      <c r="D13" s="104">
+        <f>Scenarios!D11</f>
+        <v/>
+      </c>
+      <c r="E13" s="104">
+        <f>Scenarios!D38</f>
+        <v/>
+      </c>
+      <c r="F13" s="104">
+        <f>Scenarios!F11</f>
+        <v/>
+      </c>
+      <c r="G13" s="104">
+        <f>Scenarios!G11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="90" t="inlineStr">
+        <is>
+          <t>§1202 Exclusion</t>
+        </is>
+      </c>
+      <c r="B14" s="104">
+        <f>Scenarios!B18</f>
+        <v/>
+      </c>
+      <c r="C14" s="104">
+        <f>Scenarios!C18</f>
+        <v/>
+      </c>
+      <c r="D14" s="104">
+        <f>Scenarios!D18</f>
+        <v/>
+      </c>
+      <c r="E14" s="104">
+        <f>Scenarios!D47</f>
+        <v/>
+      </c>
+      <c r="F14" s="104">
+        <f>Scenarios!F18</f>
+        <v/>
+      </c>
+      <c r="G14" s="104">
+        <f>Scenarios!G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="90" t="inlineStr">
+        <is>
+          <t>Total Tax</t>
+        </is>
+      </c>
+      <c r="B15" s="104">
+        <f>Scenarios!B24</f>
+        <v/>
+      </c>
+      <c r="C15" s="104">
+        <f>Scenarios!C24</f>
+        <v/>
+      </c>
+      <c r="D15" s="104">
+        <f>Scenarios!D24</f>
+        <v/>
+      </c>
+      <c r="E15" s="104">
+        <f>Scenarios!D49</f>
+        <v/>
+      </c>
+      <c r="F15" s="104">
+        <f>Scenarios!F24</f>
+        <v/>
+      </c>
+      <c r="G15" s="104">
+        <f>Scenarios!G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="90" t="inlineStr">
+        <is>
+          <t>Net After-Tax</t>
+        </is>
+      </c>
+      <c r="B16" s="104">
+        <f>Scenarios!B26</f>
+        <v/>
+      </c>
+      <c r="C16" s="104">
+        <f>Scenarios!C26</f>
+        <v/>
+      </c>
+      <c r="D16" s="104">
+        <f>Scenarios!D26</f>
+        <v/>
+      </c>
+      <c r="E16" s="104">
+        <f>Scenarios!D50</f>
+        <v/>
+      </c>
+      <c r="F16" s="104">
+        <f>Scenarios!F26</f>
+        <v/>
+      </c>
+      <c r="G16" s="104">
+        <f>Scenarios!G26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="90" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+      <c r="B17" s="105">
+        <f>Scenarios!B27</f>
+        <v/>
+      </c>
+      <c r="C17" s="105">
+        <f>Scenarios!C27</f>
+        <v/>
+      </c>
+      <c r="D17" s="105">
+        <f>Scenarios!D27</f>
+        <v/>
+      </c>
+      <c r="E17" s="105" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="F17" s="105">
+        <f>Scenarios!F27</f>
+        <v/>
+      </c>
+      <c r="G17" s="105">
+        <f>Scenarios!G27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="84" t="inlineStr">
+        <is>
+          <t>SENSITIVITY ANALYSIS: LBRX Price vs Tax Treatment</t>
+        </is>
+      </c>
+      <c r="B20" s="108" t="n"/>
+      <c r="C20" s="108" t="n"/>
+      <c r="D20" s="108" t="n"/>
+      <c r="E20" s="108" t="n"/>
+      <c r="F20" s="108" t="n"/>
+      <c r="G20" s="109" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="90" t="inlineStr">
+        <is>
+          <t>Tax Treatment</t>
+        </is>
+      </c>
+      <c r="B21" s="106" t="inlineStr">
+        <is>
+          <t>$5</t>
+        </is>
+      </c>
+      <c r="C21" s="106" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="D21" s="106" t="inlineStr">
+        <is>
+          <t>$15</t>
+        </is>
+      </c>
+      <c r="E21" s="106" t="inlineStr">
+        <is>
+          <t>$20</t>
+        </is>
+      </c>
+      <c r="F21" s="106" t="inlineStr">
+        <is>
+          <t>$30</t>
+        </is>
+      </c>
+      <c r="G21" s="106" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
+      </c>
+      <c r="H21" s="106" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="90" t="inlineStr">
+        <is>
+          <t>No QSBS (standard LTCG)</t>
+        </is>
+      </c>
+      <c r="B22" s="107">
+        <f>serb_shares*5-(serb_shares*5-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+      <c r="C22" s="107">
+        <f>serb_shares*10-(serb_shares*10-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+      <c r="D22" s="107">
+        <f>serb_shares*15-(serb_shares*15-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+      <c r="E22" s="107">
+        <f>serb_shares*20-(serb_shares*20-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+      <c r="F22" s="107">
+        <f>serb_shares*30-(serb_shares*30-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+      <c r="G22" s="107">
+        <f>serb_shares*50-(serb_shares*50-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+      <c r="H22" s="107">
+        <f>serb_shares*100-(serb_shares*100-serb_basis)*combined_rate</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="90" t="inlineStr">
+        <is>
+          <t>QSBS §1202 Excluded</t>
+        </is>
+      </c>
+      <c r="B23" s="107">
+        <f>serb_shares*5-MAX(0,(serb_shares*5-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+      <c r="C23" s="107">
+        <f>serb_shares*10-MAX(0,(serb_shares*10-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+      <c r="D23" s="107">
+        <f>serb_shares*15-MAX(0,(serb_shares*15-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+      <c r="E23" s="107">
+        <f>serb_shares*20-MAX(0,(serb_shares*20-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+      <c r="F23" s="107">
+        <f>serb_shares*30-MAX(0,(serb_shares*30-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+      <c r="G23" s="107">
+        <f>serb_shares*50-MAX(0,(serb_shares*50-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+      <c r="H23" s="107">
+        <f>serb_shares*100-MAX(0,(serb_shares*100-serb_basis-10000000))*combined_rate</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="119" t="inlineStr">
+        <is>
+          <t>AFTER-TAX IRR COMPARISON</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="120" t="n"/>
+      <c r="B27" s="120" t="n"/>
+      <c r="C27" s="120" t="n"/>
+      <c r="D27" s="120" t="n"/>
+      <c r="E27" s="120" t="n"/>
+      <c r="F27" s="120" t="n"/>
+      <c r="G27" s="120" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="149" t="inlineStr"/>
+      <c r="B28" s="149" t="inlineStr">
+        <is>
+          <t>S1: Lock-Up</t>
+        </is>
+      </c>
+      <c r="C28" s="149" t="inlineStr">
+        <is>
+          <t>S2: Ph3+</t>
+        </is>
+      </c>
+      <c r="D28" s="149" t="inlineStr">
+        <is>
+          <t>S3: Ph3-</t>
+        </is>
+      </c>
+      <c r="E28" s="149" t="inlineStr">
+        <is>
+          <t>S4: Dual</t>
+        </is>
+      </c>
+      <c r="F28" s="149" t="inlineStr">
+        <is>
+          <t>S5: Eve Ph2+</t>
+        </is>
+      </c>
+      <c r="G28" s="149" t="inlineStr">
+        <is>
+          <t>S6: Eve Ph2-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="89" t="inlineStr">
+        <is>
+          <t>Investment Date</t>
+        </is>
+      </c>
+      <c r="B29" s="163">
+        <f>serb_date</f>
+        <v/>
+      </c>
+      <c r="C29" s="163">
+        <f>serb_date</f>
+        <v/>
+      </c>
+      <c r="D29" s="163">
+        <f>serb_date</f>
+        <v/>
+      </c>
+      <c r="E29" s="163">
+        <f>serb_date</f>
+        <v/>
+      </c>
+      <c r="F29" s="163">
+        <f>serb_date</f>
+        <v/>
+      </c>
+      <c r="G29" s="163">
+        <f>serb_date</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="89" t="inlineStr">
+        <is>
+          <t>Exit Date</t>
+        </is>
+      </c>
+      <c r="B30" s="163">
+        <f>lockup_date</f>
+        <v/>
+      </c>
+      <c r="C30" s="163">
+        <f>ph3_date</f>
+        <v/>
+      </c>
+      <c r="D30" s="163">
+        <f>ph3_date</f>
+        <v/>
+      </c>
+      <c r="E30" s="163">
+        <f>lockup_date</f>
+        <v/>
+      </c>
+      <c r="F30" s="163">
+        <f>evecxia_ph2_date</f>
+        <v/>
+      </c>
+      <c r="G30" s="163">
+        <f>evecxia_ph2_date</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="89" t="inlineStr">
+        <is>
+          <t>Holding Period (years)</t>
+        </is>
+      </c>
+      <c r="B31" s="164">
+        <f>(B30-B29)/365.25</f>
+        <v/>
+      </c>
+      <c r="C31" s="164">
+        <f>(C30-C29)/365.25</f>
+        <v/>
+      </c>
+      <c r="D31" s="164">
+        <f>(D30-D29)/365.25</f>
+        <v/>
+      </c>
+      <c r="E31" s="164">
+        <f>(E30-E29)/365.25</f>
+        <v/>
+      </c>
+      <c r="F31" s="164">
+        <f>(F30-F29)/365.25</f>
+        <v/>
+      </c>
+      <c r="G31" s="164">
+        <f>(G30-G29)/365.25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="89" t="inlineStr">
+        <is>
+          <t>Cost Basis</t>
+        </is>
+      </c>
+      <c r="B32" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+      <c r="C32" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+      <c r="D32" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+      <c r="E32" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+      <c r="F32" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+      <c r="G32" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="89" t="inlineStr">
+        <is>
+          <t>Net After-Tax</t>
+        </is>
+      </c>
+      <c r="B33" s="107">
+        <f>Scenarios!B21</f>
+        <v/>
+      </c>
+      <c r="C33" s="107">
+        <f>Scenarios!C21</f>
+        <v/>
+      </c>
+      <c r="D33" s="107">
+        <f>Scenarios!D21</f>
+        <v/>
+      </c>
+      <c r="E33" s="107">
+        <f>Scenarios!E21</f>
+        <v/>
+      </c>
+      <c r="F33" s="107">
+        <f>Scenarios!F21</f>
+        <v/>
+      </c>
+      <c r="G33" s="107">
+        <f>Scenarios!G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="126" t="inlineStr">
+        <is>
+          <t>After-Tax IRR (annualized)</t>
+        </is>
+      </c>
+      <c r="B34" s="165">
+        <f>IF(B33&gt;0,(B33/B32)^(1/B31)-1,-1)</f>
+        <v/>
+      </c>
+      <c r="C34" s="165">
+        <f>IF(C33&gt;0,(C33/C32)^(1/C31)-1,-1)</f>
+        <v/>
+      </c>
+      <c r="D34" s="165">
+        <f>IF(D33&gt;0,(D33/D32)^(1/D31)-1,-1)</f>
+        <v/>
+      </c>
+      <c r="E34" s="165">
+        <f>IF(E33&gt;0,(E33/E32)^(1/E31)-1,-1)</f>
+        <v/>
+      </c>
+      <c r="F34" s="165">
+        <f>IF(F33&gt;0,(F33/F32)^(1/F31)-1,-1)</f>
+        <v/>
+      </c>
+      <c r="G34" s="165">
+        <f>IF(G33&gt;0,(G33/G32)^(1/G31)-1,-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="166" t="inlineStr">
+        <is>
+          <t>Note: IRR assumes single lump-sum in/out. Negative returns shown as -100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="119" t="inlineStr">
+        <is>
+          <t>2D SENSITIVITY: P(Ph2+) × EVECXIA POST-DATA VALUATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="139" t="inlineStr">
+        <is>
+          <t>Investor Net After-Tax ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="167" t="inlineStr">
+        <is>
+          <t>P(Ph2+) ↓  /  Valuation →</t>
+        </is>
+      </c>
+      <c r="B40" s="168" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="C40" s="168" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="D40" s="168" t="n">
+        <v>800000000</v>
+      </c>
+      <c r="E40" s="168" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F40" s="168" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="G40" s="168" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="H40" s="168" t="n">
+        <v>3000000000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="169" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B41" s="107">
+        <f>$A41*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C41" s="107">
+        <f>$A41*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D41" s="107">
+        <f>$A41*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E41" s="107">
+        <f>$A41*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F41" s="107">
+        <f>$A41*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G41" s="107">
+        <f>$A41*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H41" s="107">
+        <f>$A41*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A41)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="169" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B42" s="107">
+        <f>$A42*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C42" s="107">
+        <f>$A42*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D42" s="107">
+        <f>$A42*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E42" s="107">
+        <f>$A42*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F42" s="107">
+        <f>$A42*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G42" s="107">
+        <f>$A42*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H42" s="107">
+        <f>$A42*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A42)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="169" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B43" s="107">
+        <f>$A43*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C43" s="107">
+        <f>$A43*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D43" s="107">
+        <f>$A43*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E43" s="107">
+        <f>$A43*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F43" s="107">
+        <f>$A43*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G43" s="107">
+        <f>$A43*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H43" s="107">
+        <f>$A43*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A43)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="169" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B44" s="107">
+        <f>$A44*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C44" s="107">
+        <f>$A44*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D44" s="107">
+        <f>$A44*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E44" s="107">
+        <f>$A44*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F44" s="107">
+        <f>$A44*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G44" s="107">
+        <f>$A44*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H44" s="107">
+        <f>$A44*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A44)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="169" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B45" s="107">
+        <f>$A45*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C45" s="107">
+        <f>$A45*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D45" s="107">
+        <f>$A45*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E45" s="107">
+        <f>$A45*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F45" s="107">
+        <f>$A45*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G45" s="107">
+        <f>$A45*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H45" s="107">
+        <f>$A45*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A45)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="169" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="B46" s="107">
+        <f>$A46*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C46" s="107">
+        <f>$A46*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D46" s="107">
+        <f>$A46*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E46" s="107">
+        <f>$A46*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F46" s="107">
+        <f>$A46*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G46" s="107">
+        <f>$A46*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H46" s="107">
+        <f>$A46*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A46)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="169" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B47" s="107">
+        <f>$A47*(B$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="C47" s="107">
+        <f>$A47*(C$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="D47" s="107">
+        <f>$A47*(D$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="E47" s="107">
+        <f>$A47*(E$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="F47" s="107">
+        <f>$A47*(F$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="G47" s="107">
+        <f>$A47*(G$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+      <c r="H47" s="107">
+        <f>$A47*(H$40*Inputs!$B$32/Inputs!$B$65)+(1-$A47)*(Inputs!$B$62*Inputs!$B$32/Inputs!$B$65)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A10:G10"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B4:B7">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"YES"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="66" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="66" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="66" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="66" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="66" t="inlineStr">
+        <is>
+          <t>Date Accessed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LBRX Current Stock Price</t>
+        </is>
+      </c>
+      <c r="C2" s="67" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/quote/LBRX/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Market Data</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LBRX IPO Announcement</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>https://www.cooley.com/news/coverage/2025/2025-09-12-lb-pharmaceuticals-announces-$285-million-upsized-ipo</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Press Release</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LBRX Phase 2 ILLUMINATE-1</t>
+        </is>
+      </c>
+      <c r="C4" s="67" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/01/26/3225570/0/en/LB-Pharmaceuticals-Initiates-Phase-2-ILLUMINATE-1-Trial-in-Bipolar-Depression-Expanding-LB-102-Development-Program.html</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Clinical Data</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LBRX PIPE Financing Feb 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="67" t="inlineStr">
+        <is>
+          <t>https://www.stocktitan.net/news/LBRX/lb-pharmaceuticals-announces-100-0-million-private-oct35p3986tv.html</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Press Release</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Karuna BMY Acquisition</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>https://news.bms.com/news/details/2023/Bristol-Myers-Squibb-Strengthens-Neuroscience-Portfolio-with-Acquisition-of-Karuna-Therapeutics/default.aspx</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Comp Valuation</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ITCI JNJ Acquisition</t>
+        </is>
+      </c>
+      <c r="C7" s="67" t="inlineStr">
+        <is>
+          <t>https://www.jnj.com/media-center/press-releases/johnson-johnson-strengthens-neuroscience-leadership-with-acquisition-of-intra-cellular-therapies-inc</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Comp Valuation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cerevel AbbVie Acquisition</t>
+        </is>
+      </c>
+      <c r="C8" s="67" t="inlineStr">
+        <is>
+          <t>https://news.abbvie.com/2023-12-06-AbbVie-to-Acquire-Cerevel-Therapeutics-in-Transformative-Transaction-to-Strengthen-Neuroscience-Pipeline</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Comp Valuation</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cerevel Emraclidine Ph2 Failure</t>
+        </is>
+      </c>
+      <c r="C9" s="67" t="inlineStr">
+        <is>
+          <t>https://news.abbvie.com/2024-11-11-AbbVie-Provides-Update-on-Phase-2-Results-for-Emraclidine-in-Schizophrenia</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Comp Valuation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IRS §1202 QSBS Rules</t>
+        </is>
+      </c>
+      <c r="C10" s="67" t="inlineStr">
+        <is>
+          <t>https://www.irs.gov/instructions/i1040sd (Schedule D instructions)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Tax Authority</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IRS §1045 Rollover Rules</t>
+        </is>
+      </c>
+      <c r="C11" s="67" t="inlineStr">
+        <is>
+          <t>https://www.irs.gov/publications/p550 (Investment Income and Expenses)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tax Authority</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3381,524 +4837,589 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="92" t="inlineStr">
-        <is>
-          <t>Sale Price/Share</t>
-        </is>
-      </c>
-      <c r="B5" s="94">
+      <c r="A5" s="89" t="inlineStr">
+        <is>
+          <t>Sale Date</t>
+        </is>
+      </c>
+      <c r="B5" s="110">
+        <f>lockup_date</f>
+        <v/>
+      </c>
+      <c r="C5" s="110">
+        <f>ph3_date</f>
+        <v/>
+      </c>
+      <c r="D5" s="110">
+        <f>ph3_date</f>
+        <v/>
+      </c>
+      <c r="E5" s="110">
+        <f>lockup_date</f>
+        <v/>
+      </c>
+      <c r="F5" s="110">
+        <f>evecxia_ph2_date</f>
+        <v/>
+      </c>
+      <c r="G5" s="110">
+        <f>evecxia_ph2_date</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="89" t="inlineStr">
+        <is>
+          <t>Sale Price / Share</t>
+        </is>
+      </c>
+      <c r="B6" s="111">
         <f>lockup_price</f>
         <v/>
       </c>
-      <c r="C5" s="94">
-        <f>Inputs!$B$53</f>
-        <v/>
-      </c>
-      <c r="D5" s="94">
-        <f>Inputs!$B$56</f>
-        <v/>
-      </c>
-      <c r="E5" s="94">
+      <c r="C6" s="111">
+        <f>Inputs!B53</f>
+        <v/>
+      </c>
+      <c r="D6" s="111">
+        <f>Inputs!B56</f>
+        <v/>
+      </c>
+      <c r="E6" s="111">
         <f>lockup_price</f>
         <v/>
       </c>
-      <c r="F5" s="94" t="inlineStr">
-        <is>
-          <t>N/A (Evecxia)</t>
-        </is>
-      </c>
-      <c r="G5" s="94" t="inlineStr">
-        <is>
-          <t>N/A (Evecxia)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="92" t="inlineStr">
-        <is>
-          <t>Shares Sold</t>
-        </is>
-      </c>
-      <c r="B6" s="95">
+      <c r="F6" s="111">
+        <f>Inputs!B59/Inputs!B65</f>
+        <v/>
+      </c>
+      <c r="G6" s="111">
+        <f>Inputs!B62/Inputs!B65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="89" t="inlineStr">
+        <is>
+          <t>Shares</t>
+        </is>
+      </c>
+      <c r="B7" s="112">
         <f>serb_shares</f>
         <v/>
       </c>
-      <c r="C6" s="95">
+      <c r="C7" s="112">
         <f>serb_shares</f>
         <v/>
       </c>
-      <c r="D6" s="95">
+      <c r="D7" s="112">
         <f>serb_shares</f>
         <v/>
       </c>
-      <c r="E6" s="95">
-        <f>serb_shares+B25</f>
-        <v/>
-      </c>
-      <c r="F6" s="95" t="inlineStr">
-        <is>
-          <t>Evecxia</t>
-        </is>
-      </c>
-      <c r="G6" s="95" t="inlineStr">
-        <is>
-          <t>Evecxia</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="92" t="inlineStr">
+      <c r="E7" s="112">
+        <f>serb_shares+IF(Inputs!B23="",0,Inputs!B25)</f>
+        <v/>
+      </c>
+      <c r="F7" s="112">
+        <f>Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="G7" s="112">
+        <f>Inputs!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="89" t="inlineStr">
         <is>
           <t>Gross Proceeds</t>
         </is>
       </c>
-      <c r="B7" s="96">
-        <f>serb_shares*lockup_price</f>
-        <v/>
-      </c>
-      <c r="C7" s="96">
-        <f>serb_shares*Inputs!$B$53</f>
-        <v/>
-      </c>
-      <c r="D7" s="96">
-        <f>serb_shares*Inputs!$B$56</f>
-        <v/>
-      </c>
-      <c r="E7" s="96">
-        <f>B9+C9</f>
-        <v/>
-      </c>
-      <c r="F7" s="96">
-        <f>Inputs!$B$65*0.0026*Inputs!$B$59</f>
-        <v/>
-      </c>
-      <c r="G7" s="96">
-        <f>Inputs!$B$65*0.0026*Inputs!$B$62</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="92" t="inlineStr">
+      <c r="B8" s="113">
+        <f>B6*B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="113">
+        <f>C6*C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="113">
+        <f>D6*D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="113">
+        <f>E6*E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="113">
+        <f>F6*F7</f>
+        <v/>
+      </c>
+      <c r="G8" s="113">
+        <f>G6*G7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="89" t="inlineStr">
         <is>
           <t>Cost Basis</t>
         </is>
       </c>
-      <c r="B8" s="96">
+      <c r="B9" s="113">
         <f>serb_basis</f>
         <v/>
       </c>
-      <c r="C8" s="96">
+      <c r="C9" s="113">
         <f>serb_basis</f>
         <v/>
       </c>
-      <c r="D8" s="96">
+      <c r="D9" s="113">
         <f>serb_basis</f>
         <v/>
       </c>
-      <c r="E8" s="96">
-        <f>serb_basis+C25</f>
-        <v/>
-      </c>
-      <c r="F8" s="96">
+      <c r="E9" s="113">
+        <f>serb_basis+IF(Inputs!B23="",0,Inputs!B23)</f>
+        <v/>
+      </c>
+      <c r="F9" s="113">
         <f>serb_basis</f>
         <v/>
       </c>
-      <c r="G8" s="96">
+      <c r="G9" s="113">
         <f>serb_basis</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="92" t="inlineStr">
-        <is>
-          <t>Gross Gain/(Loss)</t>
-        </is>
-      </c>
-      <c r="B9" s="96">
-        <f>B9-B10</f>
-        <v/>
-      </c>
-      <c r="C9" s="96">
-        <f>C9-C10</f>
-        <v/>
-      </c>
-      <c r="D9" s="96">
-        <f>D9-D10</f>
-        <v/>
-      </c>
-      <c r="E9" s="96">
-        <f>E9-E10</f>
-        <v/>
-      </c>
-      <c r="F9" s="96">
-        <f>F9-F10</f>
-        <v/>
-      </c>
-      <c r="G9" s="96">
-        <f>G9-G10</f>
-        <v/>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="37" t="inlineStr"/>
-      <c r="B10" s="28" t="inlineStr"/>
-      <c r="C10" s="28" t="inlineStr"/>
-      <c r="D10" s="28" t="inlineStr"/>
-      <c r="E10" s="28" t="inlineStr"/>
-      <c r="F10" s="28" t="inlineStr"/>
-      <c r="G10" s="28" t="inlineStr"/>
+      <c r="A10" s="89" t="inlineStr">
+        <is>
+          <t>Gross Gain</t>
+        </is>
+      </c>
+      <c r="B10" s="113">
+        <f>B8-B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="113">
+        <f>C8-C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="113">
+        <f>D8-D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="113">
+        <f>E8-E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="113">
+        <f>F8-F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="113">
+        <f>G8-G9</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="92" t="inlineStr">
+      <c r="A11" s="89" t="inlineStr">
         <is>
           <t>Holding Period (days)</t>
         </is>
       </c>
-      <c r="B11" s="95">
+      <c r="B11" s="112">
         <f>lockup_date-serb_date</f>
         <v/>
       </c>
-      <c r="C11" s="95">
+      <c r="C11" s="112">
         <f>ph3_date-serb_date</f>
         <v/>
       </c>
-      <c r="D11" s="95">
+      <c r="D11" s="112">
         <f>ph3_date-serb_date</f>
         <v/>
       </c>
-      <c r="E11" s="95" t="inlineStr">
-        <is>
-          <t>Varies</t>
-        </is>
-      </c>
-      <c r="F11" s="95">
+      <c r="E11" s="112">
+        <f>lockup_date-serb_date</f>
+        <v/>
+      </c>
+      <c r="F11" s="112">
         <f>evecxia_ph2_date-serb_date</f>
         <v/>
       </c>
-      <c r="G11" s="95">
+      <c r="G11" s="112">
         <f>evecxia_ph2_date-serb_date</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="92" t="inlineStr">
+      <c r="A12" s="89" t="inlineStr">
         <is>
           <t>Holding Period (years)</t>
         </is>
       </c>
-      <c r="B12" s="97">
-        <f>B13/365.25</f>
-        <v/>
-      </c>
-      <c r="C12" s="97">
-        <f>C13/365.25</f>
-        <v/>
-      </c>
-      <c r="D12" s="97">
-        <f>D13/365.25</f>
-        <v/>
-      </c>
-      <c r="E12" s="97" t="inlineStr">
-        <is>
-          <t>Varies</t>
-        </is>
-      </c>
-      <c r="F12" s="97">
-        <f>F13/365.25</f>
-        <v/>
-      </c>
-      <c r="G12" s="97">
-        <f>G13/365.25</f>
+      <c r="B12" s="114">
+        <f>B11/365.25</f>
+        <v/>
+      </c>
+      <c r="C12" s="114">
+        <f>C11/365.25</f>
+        <v/>
+      </c>
+      <c r="D12" s="114">
+        <f>D11/365.25</f>
+        <v/>
+      </c>
+      <c r="E12" s="114">
+        <f>E11/365.25</f>
+        <v/>
+      </c>
+      <c r="F12" s="114">
+        <f>F11/365.25</f>
+        <v/>
+      </c>
+      <c r="G12" s="114">
+        <f>G11/365.25</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="92" t="inlineStr">
+      <c r="A13" s="89" t="inlineStr">
         <is>
           <t>Long-Term?</t>
         </is>
       </c>
-      <c r="B13" s="98">
-        <f>IF(B13&gt;365,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="C13" s="98">
-        <f>IF(C13&gt;365,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="D13" s="98">
-        <f>IF(D13&gt;365,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="E13" s="98" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F13" s="98" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="G13" s="98" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
+      <c r="B13" s="115">
+        <f>IF(B11&gt;365,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="C13" s="115">
+        <f>IF(C11&gt;365,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="D13" s="115">
+        <f>IF(D11&gt;365,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="E13" s="115">
+        <f>IF(E11&gt;365,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="F13" s="115">
+        <f>IF(F11&gt;365,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="G13" s="115">
+        <f>IF(G11&gt;365,"YES","NO")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="92" t="inlineStr">
+      <c r="A14" s="89" t="inlineStr">
         <is>
           <t>QSBS 5-Year Met?</t>
         </is>
       </c>
-      <c r="B14" s="98">
-        <f>IF(B13&gt;=1826,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="C14" s="98">
-        <f>IF(C13&gt;=1826,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="D14" s="98">
-        <f>IF(D13&gt;=1826,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="E14" s="98" t="inlineStr">
-        <is>
-          <t>See detail</t>
-        </is>
-      </c>
-      <c r="F14" s="98">
-        <f>IF(F13&gt;=1826,"YES","NO")</f>
-        <v/>
-      </c>
-      <c r="G14" s="98">
-        <f>IF(G13&gt;=1826,"YES","NO")</f>
+      <c r="B14" s="115">
+        <f>IF(AND(B11&gt;=1826,Inputs!B18="YES"),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="C14" s="115">
+        <f>IF(AND(C11&gt;=1826,Inputs!B18="YES"),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="D14" s="115">
+        <f>IF(AND(D11&gt;=1826,Inputs!B18="YES"),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="E14" s="115">
+        <f>IF(AND(E11&gt;=1826,Inputs!B18="YES"),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="F14" s="115">
+        <f>IF(AND(F11&gt;=1826,Inputs!B33="YES"),"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="G14" s="115">
+        <f>IF(AND(G11&gt;=1826,Inputs!B33="YES"),"YES","NO")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="37" t="inlineStr"/>
-      <c r="B15" s="28" t="inlineStr"/>
-      <c r="C15" s="28" t="inlineStr"/>
-      <c r="D15" s="28" t="inlineStr"/>
-      <c r="E15" s="28" t="inlineStr"/>
-      <c r="F15" s="28" t="inlineStr"/>
-      <c r="G15" s="28" t="inlineStr"/>
+      <c r="A15" s="89" t="inlineStr">
+        <is>
+          <t>§1202 Exclusion</t>
+        </is>
+      </c>
+      <c r="B15" s="113">
+        <f>IF(B14="YES",MIN(B10,MAX(10000000,10*B9)),0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="113">
+        <f>IF(C14="YES",MIN(C10,MAX(10000000,10*C9)),0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="113">
+        <f>IF(D14="YES",MIN(MAX(0,D10),MAX(10000000,10*D9)),0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="113">
+        <f>IF(E14="YES",MIN(serb_shares*lockup_price-serb_basis,MAX(10000000,10*serb_basis)),0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="113">
+        <f>IF(F14="YES",MIN(F10,MAX(10000000,10*F9)),0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="113">
+        <f>IF(G14="YES",MIN(MAX(0,G10),MAX(10000000,10*G9)),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="92" t="inlineStr">
-        <is>
-          <t>§1202 Exclusion Amount</t>
-        </is>
-      </c>
-      <c r="B16" s="96">
-        <f>IF(B16="YES",MIN(B11,10000000),0)</f>
-        <v/>
-      </c>
-      <c r="C16" s="96">
-        <f>IF(C16="YES",MIN(C11,10000000),0)</f>
-        <v/>
-      </c>
-      <c r="D16" s="96">
-        <f>IF(D16="YES",MAX(0,MIN(D11,10000000)),0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="96" t="inlineStr">
-        <is>
-          <t>See detail</t>
-        </is>
-      </c>
-      <c r="F16" s="96">
-        <f>IF(F16="YES",MIN(F11,10000000),0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="96">
-        <f>IF(G16="YES",MIN(MAX(0,G11),10000000),0)</f>
+      <c r="A16" s="89" t="inlineStr">
+        <is>
+          <t>§1045 Deferral</t>
+        </is>
+      </c>
+      <c r="B16" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="113">
+        <f>serb_shares*lockup_price-serb_basis</f>
+        <v/>
+      </c>
+      <c r="G16" s="113">
+        <f>serb_shares*lockup_price-serb_basis</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="92" t="inlineStr">
-        <is>
-          <t>§1045 Deferred Gain</t>
-        </is>
-      </c>
-      <c r="B17" s="96" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C17" s="96" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D17" s="96" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E17" s="96" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F17" s="96">
-        <f>B11</f>
-        <v/>
-      </c>
-      <c r="G17" s="96">
-        <f>B11</f>
+      <c r="A17" s="89" t="inlineStr">
+        <is>
+          <t>Taxable Gain</t>
+        </is>
+      </c>
+      <c r="B17" s="113">
+        <f>MAX(0,B10-B15-B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="113">
+        <f>MAX(0,C10-C15-C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="113">
+        <f>MAX(0,D10-D15-D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="113">
+        <f>MAX(0,E10-E15-E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="113">
+        <f>MAX(0,F10-F15)</f>
+        <v/>
+      </c>
+      <c r="G17" s="113">
+        <f>MAX(0,G10-G15)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="92" t="inlineStr">
-        <is>
-          <t>Taxable Gain</t>
-        </is>
-      </c>
-      <c r="B18" s="96">
-        <f>MAX(0,B11-B18-B19)</f>
-        <v/>
-      </c>
-      <c r="C18" s="96">
-        <f>MAX(0,C11-C18-C19)</f>
-        <v/>
-      </c>
-      <c r="D18" s="96">
-        <f>MAX(0,D11-D18-D19)</f>
-        <v/>
-      </c>
-      <c r="E18" s="96" t="inlineStr">
-        <is>
-          <t>See detail</t>
-        </is>
-      </c>
-      <c r="F18" s="96">
-        <f>MAX(0,F11-F18-F19)</f>
-        <v/>
-      </c>
-      <c r="G18" s="96">
-        <f>MAX(0,G11-G18-G19)</f>
+      <c r="A18" s="89" t="inlineStr">
+        <is>
+          <t>Federal Tax</t>
+        </is>
+      </c>
+      <c r="B18" s="113">
+        <f>IF(B13="YES",B17*eff_fed_rate,B17*Inputs!B11)</f>
+        <v/>
+      </c>
+      <c r="C18" s="113">
+        <f>IF(C13="YES",C17*eff_fed_rate,C17*Inputs!B11)</f>
+        <v/>
+      </c>
+      <c r="D18" s="113">
+        <f>IF(D13="YES",D17*eff_fed_rate,D17*Inputs!B11)</f>
+        <v/>
+      </c>
+      <c r="E18" s="113">
+        <f>IF(E13="YES",E17*eff_fed_rate,E17*Inputs!B11)</f>
+        <v/>
+      </c>
+      <c r="F18" s="113">
+        <f>IF(F13="YES",F17*eff_fed_rate,F17*Inputs!B11)</f>
+        <v/>
+      </c>
+      <c r="G18" s="113">
+        <f>IF(G13="YES",G17*eff_fed_rate,G17*Inputs!B11)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="37" t="inlineStr"/>
-      <c r="B19" s="28" t="inlineStr"/>
-      <c r="C19" s="28" t="inlineStr"/>
-      <c r="D19" s="28" t="inlineStr"/>
-      <c r="E19" s="28" t="inlineStr"/>
-      <c r="F19" s="28" t="inlineStr"/>
-      <c r="G19" s="28" t="inlineStr"/>
+      <c r="A19" s="89" t="inlineStr">
+        <is>
+          <t>State Tax</t>
+        </is>
+      </c>
+      <c r="B19" s="113">
+        <f>B17*state_rate</f>
+        <v/>
+      </c>
+      <c r="C19" s="113">
+        <f>C17*state_rate</f>
+        <v/>
+      </c>
+      <c r="D19" s="113">
+        <f>D17*state_rate</f>
+        <v/>
+      </c>
+      <c r="E19" s="113">
+        <f>E17*state_rate</f>
+        <v/>
+      </c>
+      <c r="F19" s="113">
+        <f>F17*state_rate</f>
+        <v/>
+      </c>
+      <c r="G19" s="113">
+        <f>G17*state_rate</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="92" t="inlineStr">
-        <is>
-          <t>Federal LTCG Tax</t>
-        </is>
-      </c>
-      <c r="B20" s="96">
-        <f>B20*eff_fed_rate</f>
-        <v/>
-      </c>
-      <c r="C20" s="96">
-        <f>C20*eff_fed_rate</f>
-        <v/>
-      </c>
-      <c r="D20" s="96">
-        <f>D20*eff_fed_rate</f>
-        <v/>
-      </c>
-      <c r="E20" s="96" t="inlineStr">
-        <is>
-          <t>See detail</t>
-        </is>
-      </c>
-      <c r="F20" s="96">
-        <f>F20*eff_fed_rate</f>
-        <v/>
-      </c>
-      <c r="G20" s="96">
-        <f>G20*eff_fed_rate</f>
+      <c r="A20" s="89" t="inlineStr">
+        <is>
+          <t>Total Tax</t>
+        </is>
+      </c>
+      <c r="B20" s="113">
+        <f>B18+B19</f>
+        <v/>
+      </c>
+      <c r="C20" s="113">
+        <f>C18+C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="113">
+        <f>D18+D19</f>
+        <v/>
+      </c>
+      <c r="E20" s="113">
+        <f>E18+E19</f>
+        <v/>
+      </c>
+      <c r="F20" s="113">
+        <f>F18+F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="113">
+        <f>G18+G19</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="92" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="B21" s="96">
-        <f>B20*state_rate</f>
-        <v/>
-      </c>
-      <c r="C21" s="96">
-        <f>C20*state_rate</f>
-        <v/>
-      </c>
-      <c r="D21" s="96">
-        <f>D20*state_rate</f>
-        <v/>
-      </c>
-      <c r="E21" s="96" t="inlineStr">
-        <is>
-          <t>See detail</t>
-        </is>
-      </c>
-      <c r="F21" s="96">
-        <f>F20*state_rate</f>
-        <v/>
-      </c>
-      <c r="G21" s="96">
-        <f>G20*state_rate</f>
+      <c r="A21" s="89" t="inlineStr">
+        <is>
+          <t>Net After-Tax</t>
+        </is>
+      </c>
+      <c r="B21" s="116">
+        <f>B8-B20</f>
+        <v/>
+      </c>
+      <c r="C21" s="116">
+        <f>C8-C20</f>
+        <v/>
+      </c>
+      <c r="D21" s="116">
+        <f>D8-D20</f>
+        <v/>
+      </c>
+      <c r="E21" s="116">
+        <f>E8-E20</f>
+        <v/>
+      </c>
+      <c r="F21" s="116">
+        <f>F8-F20</f>
+        <v/>
+      </c>
+      <c r="G21" s="116">
+        <f>G8-G20</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="92" t="inlineStr">
-        <is>
-          <t>Total Tax</t>
-        </is>
-      </c>
-      <c r="B22" s="96">
-        <f>B22+B23</f>
-        <v/>
-      </c>
-      <c r="C22" s="96">
-        <f>C22+C23</f>
-        <v/>
-      </c>
-      <c r="D22" s="96">
-        <f>D22+D23</f>
-        <v/>
-      </c>
-      <c r="E22" s="96" t="inlineStr">
-        <is>
-          <t>See detail</t>
-        </is>
-      </c>
-      <c r="F22" s="96">
-        <f>F22+F23</f>
-        <v/>
-      </c>
-      <c r="G22" s="96">
-        <f>G22+G23</f>
+      <c r="A22" s="89" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+      <c r="B22" s="117">
+        <f>B21/B9</f>
+        <v/>
+      </c>
+      <c r="C22" s="117">
+        <f>C21/C9</f>
+        <v/>
+      </c>
+      <c r="D22" s="117">
+        <f>D21/D9</f>
+        <v/>
+      </c>
+      <c r="E22" s="117">
+        <f>E21/E9</f>
+        <v/>
+      </c>
+      <c r="F22" s="117">
+        <f>F21/F9</f>
+        <v/>
+      </c>
+      <c r="G22" s="117">
+        <f>G21/G9</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="37" t="inlineStr"/>
-      <c r="B23" s="28" t="inlineStr"/>
-      <c r="C23" s="28" t="inlineStr"/>
-      <c r="D23" s="28" t="inlineStr"/>
-      <c r="E23" s="28" t="inlineStr"/>
-      <c r="F23" s="28" t="inlineStr"/>
-      <c r="G23" s="28" t="inlineStr"/>
+      <c r="A23" s="89" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="B23" s="118">
+        <f>IF(B10&gt;0,B20/B10,0)</f>
+        <v/>
+      </c>
+      <c r="C23" s="118">
+        <f>IF(C10&gt;0,C20/C10,0)</f>
+        <v/>
+      </c>
+      <c r="D23" s="118">
+        <f>IF(D10&gt;0,D20/D10,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="118">
+        <f>IF(E10&gt;0,E20/E10,0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="118">
+        <f>IF(F10&gt;0,F20/F10,0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="118">
+        <f>IF(G10&gt;0,G20/G10,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="92" t="inlineStr">
@@ -5633,454 +7154,948 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="68" t="inlineStr">
-        <is>
-          <t>OUTPUTS DASHBOARD</t>
+      <c r="A1" s="119" t="inlineStr">
+        <is>
+          <t>DECISION MATRIX — PROBABILITY-WEIGHTED ANALYSIS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="84" t="inlineStr">
-        <is>
-          <t>KEY FLAGS</t>
-        </is>
-      </c>
-      <c r="B3" s="108" t="n"/>
-      <c r="C3" s="109" t="n"/>
+      <c r="A3" s="120" t="inlineStr">
+        <is>
+          <t>CLINICAL PROBABILITY ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="B3" s="120" t="n"/>
+      <c r="C3" s="120" t="n"/>
+      <c r="D3" s="120" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="90" t="inlineStr">
         <is>
-          <t>QSBS 5-year met at lock-up?</t>
-        </is>
-      </c>
-      <c r="B4" s="102">
-        <f>IF(lockup_date&gt;=qsbs_5yr_date,"YES","NO")</f>
-        <v/>
+          <t>P(LBRX Phase 3 Success)</t>
+        </is>
+      </c>
+      <c r="B4" s="121" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C4" s="122" t="inlineStr">
+        <is>
+          <t>← Adjustable input (industry avg MDD Ph3: 50-60%)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="90" t="inlineStr">
         <is>
-          <t>QSBS 5-year met at Phase 3 readout?</t>
-        </is>
-      </c>
-      <c r="B5" s="102">
-        <f>IF(ph3_date&gt;=qsbs_5yr_date,"YES","NO")</f>
+          <t>P(LBRX Phase 3 Failure)</t>
+        </is>
+      </c>
+      <c r="B5" s="123">
+        <f>1-B4</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="90" t="inlineStr">
-        <is>
-          <t>§1045 eligible?</t>
-        </is>
-      </c>
-      <c r="B6" s="102">
-        <f>IF(AND((lockup_date-serb_date)&gt;180,Inputs!$B$33="YES"),"YES","NO")</f>
-        <v/>
-      </c>
+      <c r="A6" s="90" t="n"/>
+      <c r="B6" s="90" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="90" t="inlineStr">
         <is>
-          <t>§1045 → §1202 chain achievable?</t>
-        </is>
-      </c>
-      <c r="B7" s="102">
-        <f>IF(AND(B6="YES",(evecxia_ph2_date-serb_date)&gt;=1826),"YES","NO")</f>
+          <t>P(Evecxia Phase 2 Success)</t>
+        </is>
+      </c>
+      <c r="B7" s="121" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C7" s="122" t="inlineStr">
+        <is>
+          <t>← Adjustable input (CNS Ph2 success rate: 30-40%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>P(Evecxia Phase 2 Failure)</t>
+        </is>
+      </c>
+      <c r="B8" s="123">
+        <f>1-B7</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>SCENARIO COMPARISON</t>
-        </is>
-      </c>
-      <c r="B10" s="108" t="n"/>
-      <c r="C10" s="108" t="n"/>
-      <c r="D10" s="108" t="n"/>
-      <c r="E10" s="108" t="n"/>
-      <c r="F10" s="108" t="n"/>
-      <c r="G10" s="109" t="n"/>
+      <c r="A10" s="120" t="inlineStr">
+        <is>
+          <t>PATH 2: HOLD LBRX THROUGH PHASE 3</t>
+        </is>
+      </c>
+      <c r="B10" s="120" t="n"/>
+      <c r="C10" s="120" t="n"/>
+      <c r="D10" s="120" t="n"/>
+      <c r="E10" s="120" t="n"/>
+      <c r="F10" s="120" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="103" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B11" s="103" t="inlineStr">
-        <is>
-          <t>S1: Lock-Up</t>
-        </is>
-      </c>
-      <c r="C11" s="103" t="inlineStr">
-        <is>
-          <t>S2: Ph3+</t>
-        </is>
-      </c>
-      <c r="D11" s="103" t="inlineStr">
-        <is>
-          <t>S3: Ph3-</t>
-        </is>
-      </c>
-      <c r="E11" s="103" t="inlineStr">
-        <is>
-          <t>S4: Dual Lot</t>
-        </is>
-      </c>
-      <c r="F11" s="103" t="inlineStr">
-        <is>
-          <t>S5: Eve+</t>
-        </is>
-      </c>
-      <c r="G11" s="103" t="inlineStr">
-        <is>
-          <t>S6: Eve-</t>
+      <c r="A11" s="124" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B11" s="124" t="inlineStr">
+        <is>
+          <t>Probability</t>
+        </is>
+      </c>
+      <c r="C11" s="124" t="inlineStr">
+        <is>
+          <t>LBRX Price</t>
+        </is>
+      </c>
+      <c r="D11" s="124" t="inlineStr">
+        <is>
+          <t>Gross Proceeds</t>
+        </is>
+      </c>
+      <c r="E11" s="124" t="inlineStr">
+        <is>
+          <t>Tax</t>
+        </is>
+      </c>
+      <c r="F11" s="124" t="inlineStr">
+        <is>
+          <t>Net After-Tax</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="90" t="inlineStr">
         <is>
-          <t>Gross Proceeds</t>
-        </is>
-      </c>
-      <c r="B12" s="104">
-        <f>Scenarios!B9</f>
-        <v/>
-      </c>
-      <c r="C12" s="104">
-        <f>Scenarios!C9</f>
-        <v/>
-      </c>
-      <c r="D12" s="104">
-        <f>Scenarios!D9</f>
-        <v/>
-      </c>
-      <c r="E12" s="104">
-        <f>Scenarios!D36</f>
-        <v/>
-      </c>
-      <c r="F12" s="104">
-        <f>Scenarios!F9</f>
-        <v/>
-      </c>
-      <c r="G12" s="104">
-        <f>Scenarios!G9</f>
+          <t>Ph3 Positive — Low ($50)</t>
+        </is>
+      </c>
+      <c r="B12" s="123">
+        <f>B4*0.25</f>
+        <v/>
+      </c>
+      <c r="C12" s="125">
+        <f>Inputs!B52</f>
+        <v/>
+      </c>
+      <c r="D12" s="107">
+        <f>C12*serb_shares</f>
+        <v/>
+      </c>
+      <c r="E12" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="107">
+        <f>D12-E12</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="90" t="inlineStr">
         <is>
-          <t>Gain</t>
-        </is>
-      </c>
-      <c r="B13" s="104">
-        <f>Scenarios!B11</f>
-        <v/>
-      </c>
-      <c r="C13" s="104">
-        <f>Scenarios!C11</f>
-        <v/>
-      </c>
-      <c r="D13" s="104">
-        <f>Scenarios!D11</f>
-        <v/>
-      </c>
-      <c r="E13" s="104">
-        <f>Scenarios!D38</f>
-        <v/>
-      </c>
-      <c r="F13" s="104">
-        <f>Scenarios!F11</f>
-        <v/>
-      </c>
-      <c r="G13" s="104">
-        <f>Scenarios!G11</f>
+          <t>Ph3 Positive — Base ($100)</t>
+        </is>
+      </c>
+      <c r="B13" s="123">
+        <f>B4*0.50</f>
+        <v/>
+      </c>
+      <c r="C13" s="125">
+        <f>Inputs!B53</f>
+        <v/>
+      </c>
+      <c r="D13" s="107">
+        <f>C13*serb_shares</f>
+        <v/>
+      </c>
+      <c r="E13" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="107">
+        <f>D13-E13</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="90" t="inlineStr">
         <is>
-          <t>§1202 Exclusion</t>
-        </is>
-      </c>
-      <c r="B14" s="104">
-        <f>Scenarios!B18</f>
-        <v/>
-      </c>
-      <c r="C14" s="104">
-        <f>Scenarios!C18</f>
-        <v/>
-      </c>
-      <c r="D14" s="104">
-        <f>Scenarios!D18</f>
-        <v/>
-      </c>
-      <c r="E14" s="104">
-        <f>Scenarios!D47</f>
-        <v/>
-      </c>
-      <c r="F14" s="104">
-        <f>Scenarios!F18</f>
-        <v/>
-      </c>
-      <c r="G14" s="104">
-        <f>Scenarios!G18</f>
+          <t>Ph3 Positive — High ($165)</t>
+        </is>
+      </c>
+      <c r="B14" s="123">
+        <f>B4*0.25</f>
+        <v/>
+      </c>
+      <c r="C14" s="125">
+        <f>Inputs!B54</f>
+        <v/>
+      </c>
+      <c r="D14" s="107">
+        <f>C14*serb_shares</f>
+        <v/>
+      </c>
+      <c r="E14" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="107">
+        <f>D14-E14</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="90" t="inlineStr">
         <is>
-          <t>Total Tax</t>
-        </is>
-      </c>
-      <c r="B15" s="104">
-        <f>Scenarios!B24</f>
-        <v/>
-      </c>
-      <c r="C15" s="104">
-        <f>Scenarios!C24</f>
-        <v/>
-      </c>
-      <c r="D15" s="104">
-        <f>Scenarios!D24</f>
-        <v/>
-      </c>
-      <c r="E15" s="104">
-        <f>Scenarios!D49</f>
-        <v/>
-      </c>
-      <c r="F15" s="104">
-        <f>Scenarios!F24</f>
-        <v/>
-      </c>
-      <c r="G15" s="104">
-        <f>Scenarios!G24</f>
+          <t>Ph3 Negative — Low ($3.30)</t>
+        </is>
+      </c>
+      <c r="B15" s="123">
+        <f>B5*0.25</f>
+        <v/>
+      </c>
+      <c r="C15" s="125">
+        <f>Inputs!B55</f>
+        <v/>
+      </c>
+      <c r="D15" s="107">
+        <f>C15*serb_shares</f>
+        <v/>
+      </c>
+      <c r="E15" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="107">
+        <f>D15-E15</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="90" t="inlineStr">
         <is>
-          <t>Net After-Tax</t>
-        </is>
-      </c>
-      <c r="B16" s="104">
-        <f>Scenarios!B26</f>
-        <v/>
-      </c>
-      <c r="C16" s="104">
-        <f>Scenarios!C26</f>
-        <v/>
-      </c>
-      <c r="D16" s="104">
-        <f>Scenarios!D26</f>
-        <v/>
-      </c>
-      <c r="E16" s="104">
-        <f>Scenarios!D50</f>
-        <v/>
-      </c>
-      <c r="F16" s="104">
-        <f>Scenarios!F26</f>
-        <v/>
-      </c>
-      <c r="G16" s="104">
-        <f>Scenarios!G26</f>
+          <t>Ph3 Negative — Base ($6.60)</t>
+        </is>
+      </c>
+      <c r="B16" s="123">
+        <f>B5*0.50</f>
+        <v/>
+      </c>
+      <c r="C16" s="125">
+        <f>Inputs!B56</f>
+        <v/>
+      </c>
+      <c r="D16" s="107">
+        <f>C16*serb_shares</f>
+        <v/>
+      </c>
+      <c r="E16" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="107">
+        <f>D16-E16</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="90" t="inlineStr">
         <is>
-          <t>MOIC</t>
-        </is>
-      </c>
-      <c r="B17" s="105">
-        <f>Scenarios!B27</f>
-        <v/>
-      </c>
-      <c r="C17" s="105">
-        <f>Scenarios!C27</f>
-        <v/>
-      </c>
-      <c r="D17" s="105">
-        <f>Scenarios!D27</f>
-        <v/>
-      </c>
-      <c r="E17" s="105" t="inlineStr">
-        <is>
-          <t>Varies</t>
-        </is>
-      </c>
-      <c r="F17" s="105">
-        <f>Scenarios!F27</f>
-        <v/>
-      </c>
-      <c r="G17" s="105">
-        <f>Scenarios!G27</f>
+          <t>Ph3 Negative — High ($11.50)</t>
+        </is>
+      </c>
+      <c r="B17" s="123">
+        <f>B5*0.25</f>
+        <v/>
+      </c>
+      <c r="C17" s="125">
+        <f>Inputs!B57</f>
+        <v/>
+      </c>
+      <c r="D17" s="107">
+        <f>C17*serb_shares</f>
+        <v/>
+      </c>
+      <c r="E17" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="107">
+        <f>D17-E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="126" t="inlineStr">
+        <is>
+          <t>PATH 2 EXPECTED VALUE</t>
+        </is>
+      </c>
+      <c r="B19" s="123">
+        <f>SUM(B12:B17)</f>
+        <v/>
+      </c>
+      <c r="C19" s="90" t="n"/>
+      <c r="D19" s="90" t="n"/>
+      <c r="E19" s="90" t="n"/>
+      <c r="F19" s="127">
+        <f>SUMPRODUCT(B12:B17,F12:F17)/SUM(B12:B17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="84" t="inlineStr">
-        <is>
-          <t>SENSITIVITY ANALYSIS: LBRX Price vs Tax Treatment</t>
-        </is>
-      </c>
-      <c r="B20" s="108" t="n"/>
-      <c r="C20" s="108" t="n"/>
-      <c r="D20" s="108" t="n"/>
-      <c r="E20" s="108" t="n"/>
-      <c r="F20" s="108" t="n"/>
-      <c r="G20" s="109" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="90" t="inlineStr">
-        <is>
-          <t>Tax Treatment</t>
-        </is>
-      </c>
-      <c r="B21" s="106" t="inlineStr">
-        <is>
-          <t>$5</t>
-        </is>
-      </c>
-      <c r="C21" s="106" t="inlineStr">
-        <is>
-          <t>$10</t>
-        </is>
-      </c>
-      <c r="D21" s="106" t="inlineStr">
-        <is>
-          <t>$15</t>
-        </is>
-      </c>
-      <c r="E21" s="106" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="F21" s="106" t="inlineStr">
-        <is>
-          <t>$30</t>
-        </is>
-      </c>
-      <c r="G21" s="106" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="H21" s="106" t="inlineStr">
-        <is>
-          <t>$100</t>
-        </is>
+      <c r="A20" s="126" t="inlineStr">
+        <is>
+          <t>PATH 2 EXPECTED MOIC</t>
+        </is>
+      </c>
+      <c r="B20" s="90" t="n"/>
+      <c r="C20" s="90" t="n"/>
+      <c r="D20" s="90" t="n"/>
+      <c r="E20" s="90" t="n"/>
+      <c r="F20" s="128">
+        <f>F19/serb_basis</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="90" t="inlineStr">
-        <is>
-          <t>No QSBS (standard LTCG)</t>
-        </is>
-      </c>
-      <c r="B22" s="107">
-        <f>serb_shares*5-(serb_shares*5-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
-      <c r="C22" s="107">
-        <f>serb_shares*10-(serb_shares*10-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
-      <c r="D22" s="107">
-        <f>serb_shares*15-(serb_shares*15-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
-      <c r="E22" s="107">
-        <f>serb_shares*20-(serb_shares*20-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
-      <c r="F22" s="107">
-        <f>serb_shares*30-(serb_shares*30-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
-      <c r="G22" s="107">
-        <f>serb_shares*50-(serb_shares*50-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
-      <c r="H22" s="107">
-        <f>serb_shares*100-(serb_shares*100-serb_basis)*combined_rate</f>
-        <v/>
-      </c>
+      <c r="A22" s="120" t="inlineStr">
+        <is>
+          <t>PATH 3: §1045 ROLL INTO EVECXIA</t>
+        </is>
+      </c>
+      <c r="B22" s="120" t="n"/>
+      <c r="C22" s="120" t="n"/>
+      <c r="D22" s="120" t="n"/>
+      <c r="E22" s="120" t="n"/>
+      <c r="F22" s="120" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="90" t="inlineStr">
-        <is>
-          <t>QSBS §1202 Excluded</t>
-        </is>
-      </c>
-      <c r="B23" s="107">
-        <f>serb_shares*5-MAX(0,(serb_shares*5-serb_basis-10000000))*combined_rate</f>
-        <v/>
-      </c>
-      <c r="C23" s="107">
-        <f>serb_shares*10-MAX(0,(serb_shares*10-serb_basis-10000000))*combined_rate</f>
-        <v/>
-      </c>
-      <c r="D23" s="107">
-        <f>serb_shares*15-MAX(0,(serb_shares*15-serb_basis-10000000))*combined_rate</f>
-        <v/>
-      </c>
-      <c r="E23" s="107">
-        <f>serb_shares*20-MAX(0,(serb_shares*20-serb_basis-10000000))*combined_rate</f>
-        <v/>
-      </c>
-      <c r="F23" s="107">
-        <f>serb_shares*30-MAX(0,(serb_shares*30-serb_basis-10000000))*combined_rate</f>
-        <v/>
-      </c>
-      <c r="G23" s="107">
-        <f>serb_shares*50-MAX(0,(serb_shares*50-serb_basis-10000000))*combined_rate</f>
-        <v/>
-      </c>
-      <c r="H23" s="107">
-        <f>serb_shares*100-MAX(0,(serb_shares*100-serb_basis-10000000))*combined_rate</f>
+      <c r="A23" s="129" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B23" s="129" t="inlineStr">
+        <is>
+          <t>Probability</t>
+        </is>
+      </c>
+      <c r="C23" s="129" t="inlineStr">
+        <is>
+          <t>Evecxia Valuation</t>
+        </is>
+      </c>
+      <c r="D23" s="129" t="inlineStr">
+        <is>
+          <t>Gross Proceeds</t>
+        </is>
+      </c>
+      <c r="E23" s="129" t="inlineStr">
+        <is>
+          <t>Tax</t>
+        </is>
+      </c>
+      <c r="F23" s="129" t="inlineStr">
+        <is>
+          <t>Net After-Tax</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="90" t="inlineStr">
+        <is>
+          <t>Ph2 Positive — Low ($800M)</t>
+        </is>
+      </c>
+      <c r="B24" s="123">
+        <f>B7*0.25</f>
+        <v/>
+      </c>
+      <c r="C24" s="130">
+        <f>Inputs!B58</f>
+        <v/>
+      </c>
+      <c r="D24" s="107">
+        <f>C24/Inputs!B65*Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="E24" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="107">
+        <f>D24-E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="90" t="inlineStr">
+        <is>
+          <t>Ph2 Positive — Base ($1.5B)</t>
+        </is>
+      </c>
+      <c r="B25" s="123">
+        <f>B7*0.50</f>
+        <v/>
+      </c>
+      <c r="C25" s="130">
+        <f>Inputs!B59</f>
+        <v/>
+      </c>
+      <c r="D25" s="107">
+        <f>C25/Inputs!B65*Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="E25" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="107">
+        <f>D25-E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="90" t="inlineStr">
+        <is>
+          <t>Ph2 Positive — High ($3B)</t>
+        </is>
+      </c>
+      <c r="B26" s="123">
+        <f>B7*0.25</f>
+        <v/>
+      </c>
+      <c r="C26" s="130">
+        <f>Inputs!B60</f>
+        <v/>
+      </c>
+      <c r="D26" s="107">
+        <f>C26/Inputs!B65*Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="E26" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="107">
+        <f>D26-E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="90" t="inlineStr">
+        <is>
+          <t>Ph2 Negative — Low ($50M)</t>
+        </is>
+      </c>
+      <c r="B27" s="123">
+        <f>B8*0.25</f>
+        <v/>
+      </c>
+      <c r="C27" s="130">
+        <f>Inputs!B61</f>
+        <v/>
+      </c>
+      <c r="D27" s="107">
+        <f>C27/Inputs!B65*Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="E27" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="107">
+        <f>D27-E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="90" t="inlineStr">
+        <is>
+          <t>Ph2 Negative — Base ($120M)</t>
+        </is>
+      </c>
+      <c r="B28" s="123">
+        <f>B8*0.50</f>
+        <v/>
+      </c>
+      <c r="C28" s="130">
+        <f>Inputs!B62</f>
+        <v/>
+      </c>
+      <c r="D28" s="107">
+        <f>C28/Inputs!B65*Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="E28" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="107">
+        <f>D28-E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="90" t="inlineStr">
+        <is>
+          <t>Ph2 Negative — High ($250M)</t>
+        </is>
+      </c>
+      <c r="B29" s="123">
+        <f>B8*0.25</f>
+        <v/>
+      </c>
+      <c r="C29" s="130">
+        <f>Inputs!B63</f>
+        <v/>
+      </c>
+      <c r="D29" s="107">
+        <f>C29/Inputs!B65*Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="E29" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="107">
+        <f>D29-E29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="126" t="inlineStr">
+        <is>
+          <t>PATH 3 EXPECTED VALUE</t>
+        </is>
+      </c>
+      <c r="B31" s="123">
+        <f>SUM(B24:B29)</f>
+        <v/>
+      </c>
+      <c r="C31" s="90" t="n"/>
+      <c r="D31" s="90" t="n"/>
+      <c r="E31" s="90" t="n"/>
+      <c r="F31" s="127">
+        <f>SUMPRODUCT(B24:B29,F24:F29)/SUM(B24:B29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="126" t="inlineStr">
+        <is>
+          <t>PATH 3 EXPECTED MOIC</t>
+        </is>
+      </c>
+      <c r="B32" s="90" t="n"/>
+      <c r="C32" s="90" t="n"/>
+      <c r="D32" s="90" t="n"/>
+      <c r="E32" s="90" t="n"/>
+      <c r="F32" s="128">
+        <f>F31/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="120" t="inlineStr">
+        <is>
+          <t>HEAD-TO-HEAD COMPARISON</t>
+        </is>
+      </c>
+      <c r="B34" s="120" t="n"/>
+      <c r="C34" s="120" t="n"/>
+      <c r="D34" s="120" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="131" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B35" s="131" t="inlineStr">
+        <is>
+          <t>Path 2: Hold LBRX</t>
+        </is>
+      </c>
+      <c r="C35" s="131" t="inlineStr">
+        <is>
+          <t>Path 3: Roll to Evecxia</t>
+        </is>
+      </c>
+      <c r="D35" s="131" t="inlineStr">
+        <is>
+          <t>Advantage</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="89" t="inlineStr">
+        <is>
+          <t>Expected Net Value</t>
+        </is>
+      </c>
+      <c r="B36" s="107">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="C36" s="107">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="D36" s="132">
+        <f>IF(C36&gt;B36,"PATH 3","PATH 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="89" t="inlineStr">
+        <is>
+          <t>Expected MOIC</t>
+        </is>
+      </c>
+      <c r="B37" s="133">
+        <f>F20</f>
+        <v/>
+      </c>
+      <c r="C37" s="133">
+        <f>F32</f>
+        <v/>
+      </c>
+      <c r="D37" s="132">
+        <f>IF(C37&gt;B37,"PATH 3","PATH 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="89" t="inlineStr">
+        <is>
+          <t>Best Case Net</t>
+        </is>
+      </c>
+      <c r="B38" s="107">
+        <f>MAX(F12:F17)</f>
+        <v/>
+      </c>
+      <c r="C38" s="107">
+        <f>MAX(F24:F29)</f>
+        <v/>
+      </c>
+      <c r="D38" s="132">
+        <f>IF(C38&gt;B38,"PATH 3","PATH 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="89" t="inlineStr">
+        <is>
+          <t>Worst Case Net</t>
+        </is>
+      </c>
+      <c r="B39" s="107">
+        <f>MIN(F12:F17)</f>
+        <v/>
+      </c>
+      <c r="C39" s="107">
+        <f>MIN(F24:F29)</f>
+        <v/>
+      </c>
+      <c r="D39" s="132">
+        <f>IF(C39&gt;B39,"PATH 2","PATH 3")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="89" t="inlineStr">
+        <is>
+          <t>P(Net &lt; Basis)</t>
+        </is>
+      </c>
+      <c r="B40" s="123">
+        <f>SUMPRODUCT((F12:F17&lt;serb_basis)*B12:B17)</f>
+        <v/>
+      </c>
+      <c r="C40" s="123">
+        <f>SUMPRODUCT((F24:F29&lt;serb_basis)*B24:B29)</f>
+        <v/>
+      </c>
+      <c r="D40" s="90">
+        <f>IF(C40&lt;B40,"PATH 3","PATH 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="89" t="inlineStr">
+        <is>
+          <t>Tax at Exit</t>
+        </is>
+      </c>
+      <c r="B41" s="90" t="inlineStr">
+        <is>
+          <t>$0 (§1202)</t>
+        </is>
+      </c>
+      <c r="C41" s="90" t="inlineStr">
+        <is>
+          <t>$0 (§1045→§1202)</t>
+        </is>
+      </c>
+      <c r="D41" s="90" t="inlineStr">
+        <is>
+          <t>TIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="89" t="inlineStr">
+        <is>
+          <t>Liquidity</t>
+        </is>
+      </c>
+      <c r="B42" s="90" t="inlineStr">
+        <is>
+          <t>Public (post-Ph3)</t>
+        </is>
+      </c>
+      <c r="C42" s="90" t="inlineStr">
+        <is>
+          <t>Private→IPO→Lock-up</t>
+        </is>
+      </c>
+      <c r="D42" s="90" t="inlineStr">
+        <is>
+          <t>PATH 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="89" t="inlineStr">
+        <is>
+          <t>EV / Risk Ratio</t>
+        </is>
+      </c>
+      <c r="B43" s="134">
+        <f>F19/ABS(MIN(F12:F17))</f>
+        <v/>
+      </c>
+      <c r="C43" s="134">
+        <f>F31/ABS(MIN(F24:F29))</f>
+        <v/>
+      </c>
+      <c r="D43" s="132">
+        <f>IF(C43&gt;B43,"PATH 3","PATH 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="120" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+      <c r="B45" s="120" t="n"/>
+      <c r="C45" s="120" t="n"/>
+      <c r="D45" s="120" t="n"/>
+      <c r="E45" s="120" t="n"/>
+      <c r="F45" s="120" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="135" t="inlineStr">
+        <is>
+          <t>EV Advantage (Path 3 - Path 2)</t>
+        </is>
+      </c>
+      <c r="B46" s="136">
+        <f>F31-F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="135" t="inlineStr">
+        <is>
+          <t>EV Multiple (Path 3 / Path 2)</t>
+        </is>
+      </c>
+      <c r="B47" s="137">
+        <f>F31/F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="135" t="inlineStr">
+        <is>
+          <t>Recommended Path</t>
+        </is>
+      </c>
+      <c r="B48" s="138">
+        <f>IF(F31&gt;F19,"PATH 3 — Roll into Evecxia","PATH 2 — Hold LBRX")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="120" t="inlineStr">
+        <is>
+          <t>SENSITIVITY: EV BY CLINICAL PROBABILITY</t>
+        </is>
+      </c>
+      <c r="B50" s="120" t="n"/>
+      <c r="C50" s="120" t="n"/>
+      <c r="D50" s="120" t="n"/>
+      <c r="E50" s="120" t="n"/>
+      <c r="F50" s="120" t="n"/>
+      <c r="G50" s="120" t="n"/>
+      <c r="H50" s="120" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="139" t="inlineStr">
+        <is>
+          <t>Path 3 Net EV at varying P(Ph2 Success):</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="140" t="inlineStr">
+        <is>
+          <t>P(Ph2 Success)</t>
+        </is>
+      </c>
+      <c r="B52" s="141" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C52" s="141" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D52" s="141" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E52" s="141" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F52" s="141" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G52" s="141" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H52" s="141" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="89" t="inlineStr">
+        <is>
+          <t>Path 3 Expected Net</t>
+        </is>
+      </c>
+      <c r="B53" s="107">
+        <f>B52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-B52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+      <c r="C53" s="107">
+        <f>C52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-C52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+      <c r="D53" s="107">
+        <f>D52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-D52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+      <c r="E53" s="107">
+        <f>E52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-E52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+      <c r="F53" s="107">
+        <f>F52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-F52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+      <c r="G53" s="107">
+        <f>G52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-G52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+      <c r="H53" s="107">
+        <f>H52*(0.25*$D$24+0.50*$D$25+0.25*$D$26)+(1-H52)*(0.25*$D$27+0.50*$D$28+0.25*$D$29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="89" t="inlineStr">
+        <is>
+          <t>Path 2 Expected Net (for comparison)</t>
+        </is>
+      </c>
+      <c r="B54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+      <c r="C54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+      <c r="D54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+      <c r="E54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+      <c r="F54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+      <c r="G54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+      <c r="H54" s="142">
+        <f>$F$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="89" t="inlineStr">
+        <is>
+          <t>Path 3 Favored?</t>
+        </is>
+      </c>
+      <c r="B55" s="115">
+        <f>IF(B53&gt;B54,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="C55" s="115">
+        <f>IF(C53&gt;C54,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="D55" s="115">
+        <f>IF(D53&gt;D54,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="E55" s="115">
+        <f>IF(E53&gt;E54,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="F55" s="115">
+        <f>IF(F53&gt;F54,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="G55" s="115">
+        <f>IF(G53&gt;G54,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="H55" s="115">
+        <f>IF(H53&gt;H54,"YES","NO")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A10:G10"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B4:B7">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"NO"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6091,291 +8106,787 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="66" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="66" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="C1" s="66" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D1" s="66" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E1" s="66" t="inlineStr">
-        <is>
-          <t>Date Accessed</t>
+      <c r="A1" s="119" t="inlineStr">
+        <is>
+          <t>BREAKEVEN ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="120" t="inlineStr">
+        <is>
+          <t>KEY QUESTION: AT WHAT EVECXIA VALUATION DOES PATH 3 = PATH 2?</t>
+        </is>
+      </c>
+      <c r="B3" s="120" t="n"/>
+      <c r="C3" s="120" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="90" t="inlineStr">
+        <is>
+          <t>Path 2 Base Case Net (LBRX Ph3+ @ $100)</t>
+        </is>
+      </c>
+      <c r="B5" s="107">
+        <f>Scenarios!C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>Investor Evecxia Shares</t>
+        </is>
+      </c>
+      <c r="B6" s="143">
+        <f>Inputs!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="90" t="inlineStr">
+        <is>
+          <t>Evecxia Total Shares at Readout</t>
+        </is>
+      </c>
+      <c r="B7" s="143">
+        <f>Inputs!B65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>Investor Ownership %</t>
+        </is>
+      </c>
+      <c r="B8" s="144">
+        <f>B6/B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="90" t="n"/>
+      <c r="B9" s="90" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="90" t="inlineStr">
+        <is>
+          <t>Breakeven Evecxia Valuation (to match Path 2 base)</t>
+        </is>
+      </c>
+      <c r="B10" s="145">
+        <f>B5/B8</f>
+        <v/>
+      </c>
+      <c r="C10" s="122" t="inlineStr">
+        <is>
+          <t>← Evecxia must be worth this much at Phase 2 readout to match LBRX Ph3+ base</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="90" t="n"/>
+      <c r="B11" s="90" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>Breakeven as Multiple of $180M IPO</t>
+        </is>
+      </c>
+      <c r="B12" s="146">
+        <f>B10/Inputs!B64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>Breakeven as Multiple of $30M Series A</t>
+        </is>
+      </c>
+      <c r="B13" s="147">
+        <f>B10/Inputs!B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="120" t="inlineStr">
+        <is>
+          <t>CAPITAL PRESERVATION: WHAT VALUATION RETURNS YOUR $100K?</t>
+        </is>
+      </c>
+      <c r="B15" s="120" t="n"/>
+      <c r="C15" s="120" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="90" t="inlineStr">
+        <is>
+          <t>Original Invested Capital</t>
+        </is>
+      </c>
+      <c r="B17" s="107">
+        <f>serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="90" t="inlineStr">
+        <is>
+          <t>Evecxia Valuation to Return $100K</t>
+        </is>
+      </c>
+      <c r="B18" s="148">
+        <f>B17/B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="90" t="inlineStr">
+        <is>
+          <t>As % of $180M IPO Valuation</t>
+        </is>
+      </c>
+      <c r="B19" s="123">
+        <f>B18/Inputs!B64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="120" t="inlineStr">
+        <is>
+          <t>SENSITIVITY: EVECXIA VALUATION → INVESTOR NET</t>
+        </is>
+      </c>
+      <c r="B21" s="120" t="n"/>
+      <c r="C21" s="120" t="n"/>
+      <c r="D21" s="120" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="149" t="inlineStr">
+        <is>
+          <t>Evecxia Valuation ($M)</t>
+        </is>
+      </c>
+      <c r="B22" s="149" t="inlineStr">
+        <is>
+          <t>Investor Gross</t>
+        </is>
+      </c>
+      <c r="C22" s="149" t="inlineStr">
+        <is>
+          <t>Tax</t>
+        </is>
+      </c>
+      <c r="D22" s="149" t="inlineStr">
+        <is>
+          <t>Investor Net</t>
+        </is>
+      </c>
+      <c r="E22" s="149" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="130" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="B23" s="107">
+        <f>A23*$B$8</f>
+        <v/>
+      </c>
+      <c r="C23" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="107">
+        <f>B23-C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="147">
+        <f>D23/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="130" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="B24" s="107">
+        <f>A24*$B$8</f>
+        <v/>
+      </c>
+      <c r="C24" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="107">
+        <f>B24-C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="147">
+        <f>D24/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="130" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="B25" s="107">
+        <f>A25*$B$8</f>
+        <v/>
+      </c>
+      <c r="C25" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="107">
+        <f>B25-C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="147">
+        <f>D25/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="150" t="n">
+        <v>180000000</v>
+      </c>
+      <c r="B26" s="151">
+        <f>A26*$B$8</f>
+        <v/>
+      </c>
+      <c r="C26" s="151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="151">
+        <f>B26-C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="147">
+        <f>D26/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="130" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="B27" s="107">
+        <f>A27*$B$8</f>
+        <v/>
+      </c>
+      <c r="C27" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="107">
+        <f>B27-C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="147">
+        <f>D27/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="130" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="B28" s="107">
+        <f>A28*$B$8</f>
+        <v/>
+      </c>
+      <c r="C28" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="107">
+        <f>B28-C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="147">
+        <f>D28/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="130" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="B29" s="107">
+        <f>A29*$B$8</f>
+        <v/>
+      </c>
+      <c r="C29" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="107">
+        <f>B29-C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="147">
+        <f>D29/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="130" t="n">
+        <v>800000000</v>
+      </c>
+      <c r="B30" s="107">
+        <f>A30*$B$8</f>
+        <v/>
+      </c>
+      <c r="C30" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="107">
+        <f>B30-C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="147">
+        <f>D30/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="130" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="B31" s="107">
+        <f>A31*$B$8</f>
+        <v/>
+      </c>
+      <c r="C31" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="107">
+        <f>B31-C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="147">
+        <f>D31/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="130" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="B32" s="107">
+        <f>A32*$B$8</f>
+        <v/>
+      </c>
+      <c r="C32" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="107">
+        <f>B32-C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="147">
+        <f>D32/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="130" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="B33" s="107">
+        <f>A33*$B$8</f>
+        <v/>
+      </c>
+      <c r="C33" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="107">
+        <f>B33-C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="147">
+        <f>D33/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="130" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="B34" s="107">
+        <f>A34*$B$8</f>
+        <v/>
+      </c>
+      <c r="C34" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="107">
+        <f>B34-C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="147">
+        <f>D34/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="119" t="inlineStr">
+        <is>
+          <t>EVECXIA DILUTION WATERFALL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>LBRX Current Stock Price</t>
-        </is>
-      </c>
-      <c r="C2" s="67" t="inlineStr">
-        <is>
-          <t>https://finance.yahoo.com/quote/LBRX/</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Market Data</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>LBRX IPO Announcement</t>
-        </is>
-      </c>
-      <c r="C3" s="67" t="inlineStr">
-        <is>
-          <t>https://www.cooley.com/news/coverage/2025/2025-09-12-lb-pharmaceuticals-announces-$285-million-upsized-ipo</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Press Release</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
+      <c r="A2" s="122" t="inlineStr">
+        <is>
+          <t>Tracking investor ownership from Series A entry through Phase 2 readout</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>LBRX Phase 2 ILLUMINATE-1</t>
-        </is>
-      </c>
-      <c r="C4" s="67" t="inlineStr">
-        <is>
-          <t>https://www.globenewswire.com/news-release/2026/01/26/3225570/0/en/LB-Pharmaceuticals-Initiates-Phase-2-ILLUMINATE-1-Trial-in-Bipolar-Depression-Expanding-LB-102-Development-Program.html</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Clinical Data</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
+      <c r="A4" s="152" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B4" s="152" t="inlineStr">
+        <is>
+          <t>Total Shares</t>
+        </is>
+      </c>
+      <c r="C4" s="152" t="inlineStr">
+        <is>
+          <t>Investor Shares</t>
+        </is>
+      </c>
+      <c r="D4" s="152" t="inlineStr">
+        <is>
+          <t>Ownership %</t>
+        </is>
+      </c>
+      <c r="E4" s="152" t="inlineStr">
+        <is>
+          <t>Implied Value of Stake</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>LBRX PIPE Financing Feb 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="67" t="inlineStr">
-        <is>
-          <t>https://www.stocktitan.net/news/LBRX/lb-pharmaceuticals-announces-100-0-million-private-oct35p3986tv.html</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Press Release</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
+      <c r="A5" s="90" t="inlineStr">
+        <is>
+          <t>Series A Close ($30M post-money)</t>
+        </is>
+      </c>
+      <c r="B5" s="143">
+        <f>Inputs!B36</f>
+        <v/>
+      </c>
+      <c r="C5" s="143">
+        <f>Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="D5" s="144">
+        <f>C5/B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="107">
+        <f>D5*Inputs!B35</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Karuna BMY Acquisition</t>
-        </is>
-      </c>
-      <c r="C6" s="67" t="inlineStr">
-        <is>
-          <t>https://news.bms.com/news/details/2023/Bristol-Myers-Squibb-Strengthens-Neuroscience-Portfolio-with-Acquisition-of-Karuna-Therapeutics/default.aspx</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Comp Valuation</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>Bridge Round (~10% dilution, est.)</t>
+        </is>
+      </c>
+      <c r="B6" s="143">
+        <f>B5/0.9</f>
+        <v/>
+      </c>
+      <c r="C6" s="143">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="D6" s="144">
+        <f>C6/B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="107">
+        <f>D6*45000000</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ITCI JNJ Acquisition</t>
-        </is>
-      </c>
-      <c r="C7" s="67" t="inlineStr">
-        <is>
-          <t>https://www.jnj.com/media-center/press-releases/johnson-johnson-strengthens-neuroscience-leadership-with-acquisition-of-intra-cellular-therapies-inc</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Comp Valuation</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
+      <c r="A7" s="90" t="inlineStr">
+        <is>
+          <t>IPO ($180M valuation)</t>
+        </is>
+      </c>
+      <c r="B7" s="143">
+        <f>B6/0.80</f>
+        <v/>
+      </c>
+      <c r="C7" s="143">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="D7" s="144">
+        <f>C7/B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="107">
+        <f>D7*Inputs!B64</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Cerevel AbbVie Acquisition</t>
-        </is>
-      </c>
-      <c r="C8" s="67" t="inlineStr">
-        <is>
-          <t>https://news.abbvie.com/2023-12-06-AbbVie-to-Acquire-Cerevel-Therapeutics-in-Transformative-Transaction-to-Strengthen-Neuroscience-Pipeline</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Comp Valuation</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Cerevel Emraclidine Ph2 Failure</t>
-        </is>
-      </c>
-      <c r="C9" s="67" t="inlineStr">
-        <is>
-          <t>https://news.abbvie.com/2024-11-11-AbbVie-Provides-Update-on-Phase-2-Results-for-Emraclidine-in-Schizophrenia</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Comp Valuation</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>At Phase 2 Readout (365M shares est.)</t>
+        </is>
+      </c>
+      <c r="B8" s="143">
+        <f>Inputs!B65</f>
+        <v/>
+      </c>
+      <c r="C8" s="143">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="D8" s="144">
+        <f>C8/B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="107" t="inlineStr">
+        <is>
+          <t>varies by scenario</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>IRS §1202 QSBS Rules</t>
-        </is>
-      </c>
-      <c r="C10" s="67" t="inlineStr">
-        <is>
-          <t>https://www.irs.gov/instructions/i1040sd (Schedule D instructions)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Tax Authority</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
+      <c r="A10" s="153" t="inlineStr">
+        <is>
+          <t>KEY INSIGHT</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>IRS §1045 Rollover Rules</t>
-        </is>
-      </c>
-      <c r="C11" s="67" t="inlineStr">
-        <is>
-          <t>https://www.irs.gov/publications/p550 (Investment Income and Expenses)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Tax Authority</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ownership dilutes from Series A to readout:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>Series A ownership</t>
+        </is>
+      </c>
+      <c r="B12" s="144">
+        <f>D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>Readout ownership</t>
+        </is>
+      </c>
+      <c r="B13" s="144">
+        <f>D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="90" t="inlineStr">
+        <is>
+          <t>Dilution (% of original ownership lost)</t>
+        </is>
+      </c>
+      <c r="B14" s="154">
+        <f>1-D8/D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="120" t="inlineStr">
+        <is>
+          <t>STAKE VALUE AT READOUT BY SCENARIO</t>
+        </is>
+      </c>
+      <c r="B16" s="120" t="n"/>
+      <c r="C16" s="120" t="n"/>
+      <c r="D16" s="120" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="149" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B17" s="149" t="inlineStr">
+        <is>
+          <t>Company Valuation</t>
+        </is>
+      </c>
+      <c r="C17" s="149" t="inlineStr">
+        <is>
+          <t>Investor Stake Value</t>
+        </is>
+      </c>
+      <c r="D17" s="149" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="155" t="inlineStr">
+        <is>
+          <t>Ph2+ Low ($800M)</t>
+        </is>
+      </c>
+      <c r="B18" s="156">
+        <f>Inputs!B58</f>
+        <v/>
+      </c>
+      <c r="C18" s="157">
+        <f>B18*$D$8</f>
+        <v/>
+      </c>
+      <c r="D18" s="158">
+        <f>C18/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="155" t="inlineStr">
+        <is>
+          <t>Ph2+ Base ($1.5B)</t>
+        </is>
+      </c>
+      <c r="B19" s="156">
+        <f>Inputs!B59</f>
+        <v/>
+      </c>
+      <c r="C19" s="157">
+        <f>B19*$D$8</f>
+        <v/>
+      </c>
+      <c r="D19" s="158">
+        <f>C19/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="155" t="inlineStr">
+        <is>
+          <t>Ph2+ High ($3B)</t>
+        </is>
+      </c>
+      <c r="B20" s="156">
+        <f>Inputs!B60</f>
+        <v/>
+      </c>
+      <c r="C20" s="157">
+        <f>B20*$D$8</f>
+        <v/>
+      </c>
+      <c r="D20" s="158">
+        <f>C20/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="159" t="inlineStr">
+        <is>
+          <t>Ph2- Low ($50M)</t>
+        </is>
+      </c>
+      <c r="B21" s="160">
+        <f>Inputs!B61</f>
+        <v/>
+      </c>
+      <c r="C21" s="161">
+        <f>B21*$D$8</f>
+        <v/>
+      </c>
+      <c r="D21" s="162">
+        <f>C21/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="159" t="inlineStr">
+        <is>
+          <t>Ph2- Base ($120M)</t>
+        </is>
+      </c>
+      <c r="B22" s="160">
+        <f>Inputs!B62</f>
+        <v/>
+      </c>
+      <c r="C22" s="161">
+        <f>B22*$D$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="162">
+        <f>C22/serb_basis</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="159" t="inlineStr">
+        <is>
+          <t>Ph2- High ($250M)</t>
+        </is>
+      </c>
+      <c r="B23" s="160">
+        <f>Inputs!B63</f>
+        <v/>
+      </c>
+      <c r="C23" s="161">
+        <f>B23*$D$8</f>
+        <v/>
+      </c>
+      <c r="D23" s="162">
+        <f>C23/serb_basis</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove directional language favoring Path 3 from model and email
Decision Matrix: removed Advantage column, VERDICT section
(Recommended Path, EV Advantage, EV Multiple), EV/Risk Ratio
row, and green font on PATH 3 cells. Renamed to Side-by-Side
Comparison. Sensitivity row relabeled neutrally.

Email: replaced "structural problem with holding" with balanced
"if you hold" framing. Added Minerva/Sage negative comps alongside
Axsome/Karuna positive comps. Added downside return (-67%) next
to upside returns. Removed "recommending" language, replaced with
"one option for your consideration." Subject line neutralized.

https://claude.ai/code/session_01F1LU9jnNeXnwBrCMYLj1kM
</commit_message>
<xml_diff>
--- a/LBRX_QSBS_Evecxia_Model.xlsx
+++ b/LBRX_QSBS_Evecxia_Model.xlsx
@@ -55,7 +55,7 @@
     <numFmt numFmtId="173" formatCode="0.0"/>
     <numFmt numFmtId="174" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -178,6 +178,7 @@
       <color rgb="00CC0000"/>
       <sz val="12"/>
     </font>
+    <font/>
   </fonts>
   <fills count="14">
     <fill>
@@ -259,7 +260,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -301,11 +302,12 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -680,6 +682,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="25" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7709,7 +7718,7 @@
     <row r="34">
       <c r="A34" s="120" t="inlineStr">
         <is>
-          <t>HEAD-TO-HEAD COMPARISON</t>
+          <t>SIDE-BY-SIDE COMPARISON</t>
         </is>
       </c>
       <c r="B34" s="120" t="n"/>
@@ -7732,11 +7741,7 @@
           <t>Path 3: Roll to Evecxia</t>
         </is>
       </c>
-      <c r="D35" s="131" t="inlineStr">
-        <is>
-          <t>Advantage</t>
-        </is>
-      </c>
+      <c r="D35" s="102" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="89" t="inlineStr">
@@ -7752,10 +7757,7 @@
         <f>F31</f>
         <v/>
       </c>
-      <c r="D36" s="132">
-        <f>IF(C36&gt;B36,"PATH 3","PATH 2")</f>
-        <v/>
-      </c>
+      <c r="D36" s="170" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="89" t="inlineStr">
@@ -7771,10 +7773,7 @@
         <f>F32</f>
         <v/>
       </c>
-      <c r="D37" s="132">
-        <f>IF(C37&gt;B37,"PATH 3","PATH 2")</f>
-        <v/>
-      </c>
+      <c r="D37" s="170" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="89" t="inlineStr">
@@ -7790,10 +7789,7 @@
         <f>MAX(F24:F29)</f>
         <v/>
       </c>
-      <c r="D38" s="132">
-        <f>IF(C38&gt;B38,"PATH 3","PATH 2")</f>
-        <v/>
-      </c>
+      <c r="D38" s="170" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="89" t="inlineStr">
@@ -7809,10 +7805,7 @@
         <f>MIN(F24:F29)</f>
         <v/>
       </c>
-      <c r="D39" s="132">
-        <f>IF(C39&gt;B39,"PATH 2","PATH 3")</f>
-        <v/>
-      </c>
+      <c r="D39" s="170" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="89" t="inlineStr">
@@ -7828,10 +7821,7 @@
         <f>SUMPRODUCT((F24:F29&lt;serb_basis)*B24:B29)</f>
         <v/>
       </c>
-      <c r="D40" s="90">
-        <f>IF(C40&lt;B40,"PATH 3","PATH 2")</f>
-        <v/>
-      </c>
+      <c r="D40" s="170" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="89" t="inlineStr">
@@ -7849,11 +7839,7 @@
           <t>$0 (§1045→§1202)</t>
         </is>
       </c>
-      <c r="D41" s="90" t="inlineStr">
-        <is>
-          <t>TIED</t>
-        </is>
-      </c>
+      <c r="D41" s="170" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="89" t="inlineStr">
@@ -7871,75 +7857,45 @@
           <t>Private→IPO→Lock-up</t>
         </is>
       </c>
-      <c r="D42" s="90" t="inlineStr">
-        <is>
-          <t>PATH 2</t>
-        </is>
-      </c>
+      <c r="D42" s="170" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="89" t="inlineStr">
-        <is>
-          <t>EV / Risk Ratio</t>
-        </is>
-      </c>
-      <c r="B43" s="134">
-        <f>F19/ABS(MIN(F12:F17))</f>
-        <v/>
-      </c>
-      <c r="C43" s="134">
-        <f>F31/ABS(MIN(F24:F29))</f>
-        <v/>
-      </c>
-      <c r="D43" s="132">
-        <f>IF(C43&gt;B43,"PATH 3","PATH 2")</f>
-        <v/>
-      </c>
+      <c r="A43" s="170" t="n"/>
+      <c r="B43" s="171" t="n"/>
+      <c r="C43" s="171" t="n"/>
+      <c r="D43" s="170" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="120" t="inlineStr">
-        <is>
-          <t>VERDICT</t>
-        </is>
-      </c>
-      <c r="B45" s="120" t="n"/>
-      <c r="C45" s="120" t="n"/>
-      <c r="D45" s="120" t="n"/>
-      <c r="E45" s="120" t="n"/>
-      <c r="F45" s="120" t="n"/>
+      <c r="A45" s="172" t="n"/>
+      <c r="B45" s="172" t="n"/>
+      <c r="C45" s="172" t="n"/>
+      <c r="D45" s="172" t="n"/>
+      <c r="E45" s="172" t="n"/>
+      <c r="F45" s="172" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="135" t="inlineStr">
-        <is>
-          <t>EV Advantage (Path 3 - Path 2)</t>
-        </is>
-      </c>
-      <c r="B46" s="136">
-        <f>F31-F19</f>
-        <v/>
-      </c>
+      <c r="A46" s="170" t="n"/>
+      <c r="B46" s="173" t="n"/>
+      <c r="C46" s="170" t="n"/>
+      <c r="D46" s="170" t="n"/>
+      <c r="E46" s="170" t="n"/>
+      <c r="F46" s="170" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="135" t="inlineStr">
-        <is>
-          <t>EV Multiple (Path 3 / Path 2)</t>
-        </is>
-      </c>
-      <c r="B47" s="137">
-        <f>F31/F19</f>
-        <v/>
-      </c>
+      <c r="A47" s="170" t="n"/>
+      <c r="B47" s="174" t="n"/>
+      <c r="C47" s="170" t="n"/>
+      <c r="D47" s="170" t="n"/>
+      <c r="E47" s="170" t="n"/>
+      <c r="F47" s="170" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="135" t="inlineStr">
-        <is>
-          <t>Recommended Path</t>
-        </is>
-      </c>
-      <c r="B48" s="138">
-        <f>IF(F31&gt;F19,"PATH 3 — Roll into Evecxia","PATH 2 — Hold LBRX")</f>
-        <v/>
-      </c>
+      <c r="A48" s="170" t="n"/>
+      <c r="B48" s="170" t="n"/>
+      <c r="C48" s="170" t="n"/>
+      <c r="D48" s="170" t="n"/>
+      <c r="E48" s="170" t="n"/>
+      <c r="F48" s="170" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="120" t="inlineStr">
@@ -7958,7 +7914,7 @@
     <row r="51">
       <c r="A51" s="139" t="inlineStr">
         <is>
-          <t>Path 3 Net EV at varying P(Ph2 Success):</t>
+          <t>Expected net at varying P(Ph2 Success):</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8019,7 @@
     <row r="55">
       <c r="A55" s="89" t="inlineStr">
         <is>
-          <t>Path 3 Favored?</t>
+          <t>Path 3 EV &gt; Path 2 EV?</t>
         </is>
       </c>
       <c r="B55" s="115">

</xml_diff>

<commit_message>
Fix Excel errors and add professional Dashboard tab
## Changes
- Fixed all #VALUE! errors in formulas
- Added professional Dashboard tab with executive summary
- Added IRR calculation to Scenarios tab
- Created simplified 1-page variant (3 tabs: Analysis, Comps, Citations)
- Validated all 289 formulas in main model - zero errors
- Validated all 39 formulas in simplified model - zero errors

## Files
- Enhanced main model with Dashboard tab
- New simplified 1-page variant for presentations
- Backup of original file
- Comprehensive changes summary document

All formulas tested and error-free.

https://claude.ai/code/session_01F1LU9jnNeXnwBrCMYLj1kM
</commit_message>
<xml_diff>
--- a/LBRX_QSBS_Evecxia_Model.xlsx
+++ b/LBRX_QSBS_Evecxia_Model.xlsx
@@ -7,17 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Timeline" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Comps" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TaxLogic" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Decision Matrix" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Breakeven" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Dilution" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Outputs" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Sources" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Timeline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Comps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scenarios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TaxLogic" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Decision Matrix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Breakeven" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dilution" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Outputs" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Sources" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="fed_ltcg_rate">Inputs!$B$5</definedName>
@@ -52,7 +53,7 @@
     <numFmt numFmtId="170" formatCode="0.000%"/>
     <numFmt numFmtId="171" formatCode="$#,##0,,&quot;M&quot;"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +132,40 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="16"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -177,6 +210,18 @@
         <bgColor rgb="002F5496"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -194,7 +239,7 @@
       <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="9">
+  <cellStyleXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -220,8 +265,21 @@
     <xf numFmtId="169" fontId="6" fillId="0" borderId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="1"/>
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="1"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1"/>
+    <xf numFmtId="4" fontId="19" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -383,8 +441,22 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="9">
+  <cellStyles count="16">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
     <cellStyle name="ib_input" xfId="1" hidden="0"/>
     <cellStyle name="ib_formula" xfId="2" hidden="0"/>
@@ -394,6 +466,13 @@
     <cellStyle name="ib_currency" xfId="6" hidden="0"/>
     <cellStyle name="ib_pct" xfId="7" hidden="0"/>
     <cellStyle name="ib_moic" xfId="8" hidden="0"/>
+    <cellStyle name="header" xfId="9" hidden="0"/>
+    <cellStyle name="subheader" xfId="10" hidden="0"/>
+    <cellStyle name="title" xfId="11" hidden="0"/>
+    <cellStyle name="currency" xfId="12" hidden="0"/>
+    <cellStyle name="currency_decimal" xfId="13" hidden="0"/>
+    <cellStyle name="percent" xfId="14" hidden="0"/>
+    <cellStyle name="number_decimal" xfId="15" hidden="0"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -782,199 +861,804 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="65" t="inlineStr">
+        <is>
+          <t>LBRX QSBS &amp; Evecxia Investment Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="66" t="inlineStr">
+        <is>
+          <t>Analysis Date: February 16, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="67" t="inlineStr">
+        <is>
+          <t>EXECUTIVE SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="68" t="inlineStr">
+        <is>
+          <t>Investment Parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Initial Investment (Series B)</t>
+        </is>
+      </c>
+      <c r="B7" s="58">
+        <f>Inputs!B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Series B Share Price</t>
+        </is>
+      </c>
+      <c r="B8" s="69">
+        <f>Inputs!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Shares Acquired</t>
+        </is>
+      </c>
+      <c r="B9" s="70">
+        <f>Inputs!B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Investment Date</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>Inputs!B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>QSBS 5-Year Date</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>Inputs!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="68" t="inlineStr">
+        <is>
+          <t>Tax Rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Federal LTCG Rate</t>
+        </is>
+      </c>
+      <c r="B14" s="56">
+        <f>Inputs!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Effective Federal Rate (incl. NIIT)</t>
+        </is>
+      </c>
+      <c r="B15" s="56">
+        <f>Inputs!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>State Tax Rate</t>
+        </is>
+      </c>
+      <c r="B16" s="56">
+        <f>Inputs!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Combined Tax Rate</t>
+        </is>
+      </c>
+      <c r="B17" s="56">
+        <f>Inputs!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>SCENARIO COMPARISON</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="71" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B22" s="71" t="inlineStr">
+        <is>
+          <t>S1: Lock-Up</t>
+        </is>
+      </c>
+      <c r="C22" s="71" t="inlineStr">
+        <is>
+          <t>S2: Ph3+</t>
+        </is>
+      </c>
+      <c r="D22" s="71" t="inlineStr">
+        <is>
+          <t>S3: Ph3-</t>
+        </is>
+      </c>
+      <c r="E22" s="71" t="inlineStr">
+        <is>
+          <t>S4: Dual Lot</t>
+        </is>
+      </c>
+      <c r="F22" s="71" t="inlineStr">
+        <is>
+          <t>S5: Eve Ph2+</t>
+        </is>
+      </c>
+      <c r="G22" s="71" t="inlineStr">
+        <is>
+          <t>S6: Eve Ph2-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="72" t="inlineStr">
+        <is>
+          <t>Sale Date</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>Scenarios!A5</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>Scenarios!B5</f>
+        <v/>
+      </c>
+      <c r="D23">
+        <f>Scenarios!C5</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>Scenarios!D5</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>Scenarios!E5</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>Scenarios!F5</f>
+        <v/>
+      </c>
+      <c r="H23">
+        <f>Scenarios!G5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="72" t="inlineStr">
+        <is>
+          <t>Sale Price/Share</t>
+        </is>
+      </c>
+      <c r="B24" s="69">
+        <f>Scenarios!A6</f>
+        <v/>
+      </c>
+      <c r="C24" s="69">
+        <f>Scenarios!B6</f>
+        <v/>
+      </c>
+      <c r="D24" s="69">
+        <f>Scenarios!C6</f>
+        <v/>
+      </c>
+      <c r="E24" s="69">
+        <f>Scenarios!D6</f>
+        <v/>
+      </c>
+      <c r="F24" s="69">
+        <f>Scenarios!E6</f>
+        <v/>
+      </c>
+      <c r="G24" s="69">
+        <f>Scenarios!F6</f>
+        <v/>
+      </c>
+      <c r="H24" s="69">
+        <f>Scenarios!G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t>Gross Proceeds</t>
+        </is>
+      </c>
+      <c r="B25" s="58">
+        <f>Scenarios!A8</f>
+        <v/>
+      </c>
+      <c r="C25" s="58">
+        <f>Scenarios!B8</f>
+        <v/>
+      </c>
+      <c r="D25" s="58">
+        <f>Scenarios!C8</f>
+        <v/>
+      </c>
+      <c r="E25" s="58">
+        <f>Scenarios!D8</f>
+        <v/>
+      </c>
+      <c r="F25" s="58">
+        <f>Scenarios!E8</f>
+        <v/>
+      </c>
+      <c r="G25" s="58">
+        <f>Scenarios!F8</f>
+        <v/>
+      </c>
+      <c r="H25" s="58">
+        <f>Scenarios!G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>Gross Gain</t>
+        </is>
+      </c>
+      <c r="B26" s="58">
+        <f>Scenarios!A10</f>
+        <v/>
+      </c>
+      <c r="C26" s="58">
+        <f>Scenarios!B10</f>
+        <v/>
+      </c>
+      <c r="D26" s="58">
+        <f>Scenarios!C10</f>
+        <v/>
+      </c>
+      <c r="E26" s="58">
+        <f>Scenarios!D10</f>
+        <v/>
+      </c>
+      <c r="F26" s="58">
+        <f>Scenarios!E10</f>
+        <v/>
+      </c>
+      <c r="G26" s="58">
+        <f>Scenarios!F10</f>
+        <v/>
+      </c>
+      <c r="H26" s="58">
+        <f>Scenarios!G10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>QSBS 5-Year Met?</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>Scenarios!A14</f>
+        <v/>
+      </c>
+      <c r="C27">
+        <f>Scenarios!B14</f>
+        <v/>
+      </c>
+      <c r="D27">
+        <f>Scenarios!C14</f>
+        <v/>
+      </c>
+      <c r="E27">
+        <f>Scenarios!D14</f>
+        <v/>
+      </c>
+      <c r="F27">
+        <f>Scenarios!E14</f>
+        <v/>
+      </c>
+      <c r="G27">
+        <f>Scenarios!F14</f>
+        <v/>
+      </c>
+      <c r="H27">
+        <f>Scenarios!G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>§1202 Exclusion</t>
+        </is>
+      </c>
+      <c r="B28" s="58">
+        <f>Scenarios!A15</f>
+        <v/>
+      </c>
+      <c r="C28" s="58">
+        <f>Scenarios!B15</f>
+        <v/>
+      </c>
+      <c r="D28" s="58">
+        <f>Scenarios!C15</f>
+        <v/>
+      </c>
+      <c r="E28" s="58">
+        <f>Scenarios!D15</f>
+        <v/>
+      </c>
+      <c r="F28" s="58">
+        <f>Scenarios!E15</f>
+        <v/>
+      </c>
+      <c r="G28" s="58">
+        <f>Scenarios!F15</f>
+        <v/>
+      </c>
+      <c r="H28" s="58">
+        <f>Scenarios!G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="72" t="inlineStr">
+        <is>
+          <t>Total Tax</t>
+        </is>
+      </c>
+      <c r="B29" s="58">
+        <f>Scenarios!A20</f>
+        <v/>
+      </c>
+      <c r="C29" s="58">
+        <f>Scenarios!B20</f>
+        <v/>
+      </c>
+      <c r="D29" s="58">
+        <f>Scenarios!C20</f>
+        <v/>
+      </c>
+      <c r="E29" s="58">
+        <f>Scenarios!D20</f>
+        <v/>
+      </c>
+      <c r="F29" s="58">
+        <f>Scenarios!E20</f>
+        <v/>
+      </c>
+      <c r="G29" s="58">
+        <f>Scenarios!F20</f>
+        <v/>
+      </c>
+      <c r="H29" s="58">
+        <f>Scenarios!G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="72" t="inlineStr">
+        <is>
+          <t>Net After-Tax</t>
+        </is>
+      </c>
+      <c r="B30" s="58">
+        <f>Scenarios!A21</f>
+        <v/>
+      </c>
+      <c r="C30" s="58">
+        <f>Scenarios!B21</f>
+        <v/>
+      </c>
+      <c r="D30" s="58">
+        <f>Scenarios!C21</f>
+        <v/>
+      </c>
+      <c r="E30" s="58">
+        <f>Scenarios!D21</f>
+        <v/>
+      </c>
+      <c r="F30" s="58">
+        <f>Scenarios!E21</f>
+        <v/>
+      </c>
+      <c r="G30" s="58">
+        <f>Scenarios!F21</f>
+        <v/>
+      </c>
+      <c r="H30" s="58">
+        <f>Scenarios!G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="72" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+      <c r="B31" s="70">
+        <f>Scenarios!A22</f>
+        <v/>
+      </c>
+      <c r="C31" s="70">
+        <f>Scenarios!B22</f>
+        <v/>
+      </c>
+      <c r="D31" s="70">
+        <f>Scenarios!C22</f>
+        <v/>
+      </c>
+      <c r="E31" s="70">
+        <f>Scenarios!D22</f>
+        <v/>
+      </c>
+      <c r="F31" s="70">
+        <f>Scenarios!E22</f>
+        <v/>
+      </c>
+      <c r="G31" s="70">
+        <f>Scenarios!F22</f>
+        <v/>
+      </c>
+      <c r="H31" s="70">
+        <f>Scenarios!G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="72" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="B32" s="56">
+        <f>Scenarios!A23</f>
+        <v/>
+      </c>
+      <c r="C32" s="56">
+        <f>Scenarios!B23</f>
+        <v/>
+      </c>
+      <c r="D32" s="56">
+        <f>Scenarios!C23</f>
+        <v/>
+      </c>
+      <c r="E32" s="56">
+        <f>Scenarios!D23</f>
+        <v/>
+      </c>
+      <c r="F32" s="56">
+        <f>Scenarios!E23</f>
+        <v/>
+      </c>
+      <c r="G32" s="56">
+        <f>Scenarios!F23</f>
+        <v/>
+      </c>
+      <c r="H32" s="56">
+        <f>Scenarios!G23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="25" customHeight="1">
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>PROBABILITY-WEIGHTED DECISION ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="73" t="inlineStr">
+        <is>
+          <t>P(LBRX Phase 3 Success)</t>
+        </is>
+      </c>
+      <c r="B37" s="56">
+        <f>"Decision Matrix"!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="73" t="inlineStr">
+        <is>
+          <t>P(Evecxia Phase 2 Success)</t>
+        </is>
+      </c>
+      <c r="B38" s="56">
+        <f>"Decision Matrix"!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="72" t="inlineStr">
+        <is>
+          <t>Path 2 Expected Value (Hold LBRX)</t>
+        </is>
+      </c>
+      <c r="B40" s="58">
+        <f>"Decision Matrix"!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="72" t="inlineStr">
+        <is>
+          <t>Path 3 Expected Value (§1045 to Evecxia)</t>
+        </is>
+      </c>
+      <c r="B41" s="58">
+        <f>"Decision Matrix"!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="73" t="inlineStr">
+        <is>
+          <t>Difference (Path 3 - Path 2)</t>
+        </is>
+      </c>
+      <c r="B42" s="58">
+        <f>"Decision Matrix"!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="25" customHeight="1">
+      <c r="A45" s="67" t="inlineStr">
+        <is>
+          <t>KEY INSIGHTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="74" t="inlineStr">
+        <is>
+          <t>• Lock-up sale (March 2026) does NOT qualify for §1202 QSBS exclusion (&lt; 5 years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="74" t="inlineStr">
+        <is>
+          <t>• QSBS 5-year threshold met on May 3, 2027 (Phase 3 scenarios qualify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="74" t="inlineStr">
+        <is>
+          <t>• §1045 rollover to Evecxia can defer gain and preserve tacked holding period</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="74" t="inlineStr">
+        <is>
+          <t>• Dual lot scenario (Series B + C) mixes QSBS-eligible and non-eligible shares</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="74" t="inlineStr">
+        <is>
+          <t>• Evecxia pathway provides upside optionality but carries binary Phase 2 risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="74" t="inlineStr">
+        <is>
+          <t>• Tax savings from §1202 can be worth $0-$238k depending on scenario and timing</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>LBRX QSBS &amp; Evecxia Scenario Model — README</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>EVECXIA DILUTION WATERFALL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>WHAT THIS MODEL DOES:</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tracking investor ownership from Series A through Phase 2 readout</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>This Excel model analyzes tax scenarios for LBRX (LB Pharmaceuticals) Series B/C investors under QSBS rules, including §1202 exclusion and §1045 rollover into Evecxia Therapeutics.</t>
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>Total Shares</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Investor Shares</t>
+        </is>
+      </c>
+      <c r="D4" s="62" t="inlineStr">
+        <is>
+          <t>Ownership %</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="inlineStr">
+        <is>
+          <t>Stake Value</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Series A Close ($30M post-money)</t>
+        </is>
+      </c>
+      <c r="B5" s="24">
+        <f>Inputs!B36</f>
+        <v/>
+      </c>
+      <c r="C5" s="24">
+        <f>Inputs!B32</f>
+        <v/>
+      </c>
+      <c r="D5" s="59">
+        <f>C5/B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="58">
+        <f>D5*Inputs!B35</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO USE:</t>
-        </is>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IPO ($180M valuation)</t>
+        </is>
+      </c>
+      <c r="B6" s="24">
+        <f>B5/0.80</f>
+        <v/>
+      </c>
+      <c r="C6" s="24">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="D6" s="59">
+        <f>C6/B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="58">
+        <f>D6*Inputs!B64</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>1. Go to the Inputs tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2. Modify investor-specific assumptions in light yellow cells:</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Federal LTCG rate, NIIT, state tax rate (rows 5-9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Series B cost basis and share price (rows 15-16)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Lock-up price (row 42) — EDITABLE to test different sale prices</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Scenario valuations (rows 52-65) — Adjust based on your comp analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>3. Review Scenarios tab for 6 tax outcome scenarios</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>4. Check Decision Matrix for probability-weighted analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>5. Review Outputs dashboard for summary comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>KEY TAX RULES EMBEDDED IN THIS MODEL:</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>• Dilution is not a taxable event; tax = sale proceeds minus basis, lot-by-lot</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>• §1202 requires 5 full years of holding; March 2026 sale of May 2022 stock = no exclusion</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>• Tranches are separate tax lots; Series B QSBS does not blend with Series C non-QSBS</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>• IPO conversion to common does not erase lot identity</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• §1045 rollover can defer gain and preserve tacked holding period if requirements met</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>IMPORTANT DISCLAIMER:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>This is an analytical model for illustrative purposes, NOT tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Consult a qualified CPA or tax attorney before making investment decisions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>§1045 rollovers have specific requirements; state tax treatment varies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>For questions or issues with this model, contact the model creator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Generated: 2026-02-14 08:23</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>At Phase 2 Readout (365M shares est.)</t>
+        </is>
+      </c>
+      <c r="B7" s="24">
+        <f>Inputs!B65</f>
+        <v/>
+      </c>
+      <c r="C7" s="24">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="D7" s="59">
+        <f>C7/B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="58" t="inlineStr">
+        <is>
+          <t>varies by scenario</t>
         </is>
       </c>
     </row>
@@ -983,7 +1667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1306,7 +1990,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1387,6 +2071,213 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LBRX QSBS &amp; Evecxia Scenario Model — README</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>WHAT THIS MODEL DOES:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>This Excel model analyzes tax scenarios for LBRX (LB Pharmaceuticals) Series B/C investors under QSBS rules, including §1202 exclusion and §1045 rollover into Evecxia Therapeutics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO USE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>1. Go to the Inputs tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2. Modify investor-specific assumptions in light yellow cells:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Federal LTCG rate, NIIT, state tax rate (rows 5-9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Series B cost basis and share price (rows 15-16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Lock-up price (row 42) — EDITABLE to test different sale prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Scenario valuations (rows 52-65) — Adjust based on your comp analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3. Review Scenarios tab for 6 tax outcome scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>4. Check Decision Matrix for probability-weighted analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>5. Review Outputs dashboard for summary comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>KEY TAX RULES EMBEDDED IN THIS MODEL:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Dilution is not a taxable event; tax = sale proceeds minus basis, lot-by-lot</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>• §1202 requires 5 full years of holding; March 2026 sale of May 2022 stock = no exclusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>• Tranches are separate tax lots; Series B QSBS does not blend with Series C non-QSBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>• IPO conversion to common does not erase lot identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>• §1045 rollover can defer gain and preserve tacked holding period if requirements met</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT DISCLAIMER:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>This is an analytical model for illustrative purposes, NOT tax advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Consult a qualified CPA or tax attorney before making investment decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>§1045 rollovers have specific requirements; state tax treatment varies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>For questions or issues with this model, contact the model creator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Generated: 2026-02-14 08:23</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1968,7 +2859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2241,7 +3132,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2378,13 +3269,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3025,6 +3916,37 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>IRR (%)</t>
+        </is>
+      </c>
+      <c r="B24" s="56">
+        <f>IF(B9&gt;0,POWER(B21/B9,1/B12)-1,0)</f>
+        <v/>
+      </c>
+      <c r="C24" s="56">
+        <f>IF(C9&gt;0,POWER(C21/C9,1/C12)-1,0)</f>
+        <v/>
+      </c>
+      <c r="D24" s="56">
+        <f>IF(D9&gt;0,POWER(D21/D9,1/D12)-1,0)</f>
+        <v/>
+      </c>
+      <c r="E24" s="56">
+        <f>IF(E9&gt;0,POWER(E21/E9,1/E12)-1,0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="56">
+        <f>IF(F9&gt;0,POWER(F21/F9,1/F12)-1,0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="56">
+        <f>IF(G9&gt;0,POWER(G21/G9,1/G12)-1,0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
@@ -3033,7 +3955,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3113,7 +4035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3256,7 +4178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3352,136 +4274,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>EVECXIA DILUTION WATERFALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Tracking investor ownership from Series A through Phase 2 readout</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="62" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="B4" s="62" t="inlineStr">
-        <is>
-          <t>Total Shares</t>
-        </is>
-      </c>
-      <c r="C4" s="62" t="inlineStr">
-        <is>
-          <t>Investor Shares</t>
-        </is>
-      </c>
-      <c r="D4" s="62" t="inlineStr">
-        <is>
-          <t>Ownership %</t>
-        </is>
-      </c>
-      <c r="E4" s="62" t="inlineStr">
-        <is>
-          <t>Stake Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Series A Close ($30M post-money)</t>
-        </is>
-      </c>
-      <c r="B5" s="24">
-        <f>Inputs!B36</f>
-        <v/>
-      </c>
-      <c r="C5" s="24">
-        <f>Inputs!B32</f>
-        <v/>
-      </c>
-      <c r="D5" s="59">
-        <f>C5/B5</f>
-        <v/>
-      </c>
-      <c r="E5" s="58">
-        <f>D5*Inputs!B35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IPO ($180M valuation)</t>
-        </is>
-      </c>
-      <c r="B6" s="24">
-        <f>B5/0.80</f>
-        <v/>
-      </c>
-      <c r="C6" s="24">
-        <f>C5</f>
-        <v/>
-      </c>
-      <c r="D6" s="59">
-        <f>C6/B6</f>
-        <v/>
-      </c>
-      <c r="E6" s="58">
-        <f>D6*Inputs!B64</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>At Phase 2 Readout (365M shares est.)</t>
-        </is>
-      </c>
-      <c r="B7" s="24">
-        <f>Inputs!B65</f>
-        <v/>
-      </c>
-      <c r="C7" s="24">
-        <f>C5</f>
-        <v/>
-      </c>
-      <c r="D7" s="59">
-        <f>C7/B7</f>
-        <v/>
-      </c>
-      <c r="E7" s="58" t="inlineStr">
-        <is>
-          <t>varies by scenario</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>